<commit_message>
Atualizacao de arquivos - 15/09/2026 12:02:13,42
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1274" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6CB8EE37-B1FF-4FAD-9517-4B8AF1B195D7}"/>
+  <xr:revisionPtr revIDLastSave="1287" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E076089F-D80F-42F5-9F72-0EE933C6F1F2}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14098" uniqueCount="2542">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14128" uniqueCount="2547">
   <si>
     <t>ID</t>
   </si>
@@ -7908,6 +7908,22 @@
   </si>
   <si>
     <t>FRQ RIBEIRAO PRETO R01</t>
+  </si>
+  <si>
+    <t>Tive uma experiência muito ruim. Sempre paguei as mensalidades da Brastemp por débito automático, portanto sempe em dia. Na passagem da Brastemp para a Culligan, houve uma mensalidade que ficou em aberto, não sei porquê. Pedi várias vezes para que me mandassem um boleto para que eu pudesse saldar essa pendência, e nunca recebi. Há duas semanas pedi uma revisão urgente porque a água do filtro estava saindo com pó preto. Me informaram que não poderiam agendar o serviço por causa da pendência de pagamento. Diante da minha indignação, finalmente me mandaram o boleto, paguei e recebi o serviço, com duas semanas de atraso. Achei a atitude muito desagradável para com uma usuária, como eu, que sempre foi pontual.</t>
+  </si>
+  <si>
+    <t>marquei manutencao e a pessoa nao apareceu. e nao ligou pra avisar
+ai marquei outro dia e. deu certo , foi bom o atendimento</t>
+  </si>
+  <si>
+    <t>tive muitos problemas para conseguir fazer essa solicitação, e só consegui após entrar no reclame aqui</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aparelho veio com defeito e até o momento não consegui contato com o suporte </t>
+  </si>
+  <si>
+    <t>Pela segunda vez foi combinado a vinda do Técnico para verificação do Purificador e não foi realizada a visita.</t>
   </si>
 </sst>
 </file>
@@ -8363,7 +8379,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1556"/>
+  <dimension ref="A1:M1561"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -67768,6 +67784,136 @@
         <v>2419</v>
       </c>
     </row>
+    <row r="1557" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1557" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1557" s="4">
+        <v>141674</v>
+      </c>
+      <c r="D1557" s="2">
+        <v>46279</v>
+      </c>
+      <c r="E1557" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1557" s="4" t="s">
+        <v>2542</v>
+      </c>
+      <c r="G1557" s="4" t="s">
+        <v>1418</v>
+      </c>
+      <c r="H1557" s="4" t="s">
+        <v>1443</v>
+      </c>
+      <c r="M1557" s="4" t="s">
+        <v>2419</v>
+      </c>
+    </row>
+    <row r="1558" spans="2:13" ht="60" x14ac:dyDescent="0.25">
+      <c r="B1558" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1558" s="4">
+        <v>135185</v>
+      </c>
+      <c r="D1558" s="2">
+        <v>46279</v>
+      </c>
+      <c r="E1558" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1558" s="5" t="s">
+        <v>2543</v>
+      </c>
+      <c r="G1558" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1558" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="M1558" s="4" t="s">
+        <v>2418</v>
+      </c>
+    </row>
+    <row r="1559" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1559" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1559" s="4">
+        <v>139941</v>
+      </c>
+      <c r="D1559" s="2">
+        <v>46279</v>
+      </c>
+      <c r="E1559" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1559" s="4" t="s">
+        <v>2544</v>
+      </c>
+      <c r="G1559" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1559" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1559" s="4" t="s">
+        <v>2494</v>
+      </c>
+    </row>
+    <row r="1560" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1560" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1560" s="4">
+        <v>143045</v>
+      </c>
+      <c r="D1560" s="2">
+        <v>46279</v>
+      </c>
+      <c r="E1560" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1560" s="4" t="s">
+        <v>2545</v>
+      </c>
+      <c r="G1560" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1560" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="M1560" s="4" t="s">
+        <v>2453</v>
+      </c>
+    </row>
+    <row r="1561" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1561" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1561" s="4">
+        <v>133539</v>
+      </c>
+      <c r="D1561" s="2">
+        <v>46280</v>
+      </c>
+      <c r="E1561" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1561" s="4" t="s">
+        <v>2546</v>
+      </c>
+      <c r="G1561" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1561" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="M1561" s="4" t="s">
+        <v>2494</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 16/09/2026 10:54:43,29
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1287" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E076089F-D80F-42F5-9F72-0EE933C6F1F2}"/>
+  <xr:revisionPtr revIDLastSave="1298" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{484A27C1-DB15-4DA9-A93B-40D3EFA25BCD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14128" uniqueCount="2547">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14146" uniqueCount="2552">
   <si>
     <t>ID</t>
   </si>
@@ -7924,6 +7924,22 @@
   </si>
   <si>
     <t>Pela segunda vez foi combinado a vinda do Técnico para verificação do Purificador e não foi realizada a visita.</t>
+  </si>
+  <si>
+    <t>O representante reclamou do serviço, tbm não deixou ficha de ordem de serviço serviço , Segunda via pra mim.</t>
+  </si>
+  <si>
+    <t>Equipamento com defeito e estou aguardando o técnico para solucionar o problema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não apareceu ninguêm nem deram uma satisfação
+</t>
+  </si>
+  <si>
+    <t>AT SJRPRETO SP R02</t>
+  </si>
+  <si>
+    <t>FRQ GALEAO SUL RJ R03</t>
   </si>
 </sst>
 </file>
@@ -8379,7 +8395,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1561"/>
+  <dimension ref="A1:M1564"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -67914,6 +67930,84 @@
         <v>2494</v>
       </c>
     </row>
+    <row r="1562" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1562" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1562" s="4">
+        <v>115696</v>
+      </c>
+      <c r="D1562" s="2">
+        <v>46280</v>
+      </c>
+      <c r="E1562" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1562" s="4" t="s">
+        <v>2547</v>
+      </c>
+      <c r="G1562" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1562" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="M1562" s="4" t="s">
+        <v>2550</v>
+      </c>
+    </row>
+    <row r="1563" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1563" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1563" s="4">
+        <v>143317</v>
+      </c>
+      <c r="D1563" s="2">
+        <v>46280</v>
+      </c>
+      <c r="E1563" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1563" s="4" t="s">
+        <v>2548</v>
+      </c>
+      <c r="G1563" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1563" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="M1563" s="4" t="s">
+        <v>2531</v>
+      </c>
+    </row>
+    <row r="1564" spans="2:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="B1564" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1564" s="4">
+        <v>117140</v>
+      </c>
+      <c r="D1564" s="2">
+        <v>46280</v>
+      </c>
+      <c r="E1564" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1564" s="5" t="s">
+        <v>2549</v>
+      </c>
+      <c r="G1564" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1564" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="M1564" s="4" t="s">
+        <v>2551</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 17/09/2026 10:14:25,95
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1298" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{484A27C1-DB15-4DA9-A93B-40D3EFA25BCD}"/>
+  <xr:revisionPtr revIDLastSave="1309" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90D3BC6C-9816-4BF1-9CBE-F34981014D58}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14146" uniqueCount="2552">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14189" uniqueCount="2556">
   <si>
     <t>ID</t>
   </si>
@@ -7940,6 +7940,18 @@
   </si>
   <si>
     <t>FRQ GALEAO SUL RJ R03</t>
+  </si>
+  <si>
+    <t>16/09/2026</t>
+  </si>
+  <si>
+    <t>purificador continua com gosto ruim</t>
+  </si>
+  <si>
+    <t>prestador não veio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prestador de serviço não compareceu </t>
   </si>
 </sst>
 </file>
@@ -8395,7 +8407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1564"/>
+  <dimension ref="A1:M1567"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -67822,6 +67834,12 @@
       <c r="H1557" s="4" t="s">
         <v>1443</v>
       </c>
+      <c r="I1557" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1557" s="4" t="s">
+        <v>1337</v>
+      </c>
       <c r="M1557" s="4" t="s">
         <v>2419</v>
       </c>
@@ -67848,6 +67866,12 @@
       <c r="H1558" s="4" t="s">
         <v>948</v>
       </c>
+      <c r="I1558" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1558" s="4" t="s">
+        <v>1337</v>
+      </c>
       <c r="M1558" s="4" t="s">
         <v>2418</v>
       </c>
@@ -67874,6 +67898,12 @@
       <c r="H1559" s="4" t="s">
         <v>21</v>
       </c>
+      <c r="I1559" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1559" s="4" t="s">
+        <v>1338</v>
+      </c>
       <c r="M1559" s="4" t="s">
         <v>2494</v>
       </c>
@@ -67900,6 +67930,12 @@
       <c r="H1560" s="4" t="s">
         <v>29</v>
       </c>
+      <c r="I1560" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1560" s="4" t="s">
+        <v>1337</v>
+      </c>
       <c r="M1560" s="4" t="s">
         <v>2453</v>
       </c>
@@ -67926,6 +67962,12 @@
       <c r="H1561" s="4" t="s">
         <v>948</v>
       </c>
+      <c r="I1561" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1561" s="4" t="s">
+        <v>1337</v>
+      </c>
       <c r="M1561" s="4" t="s">
         <v>2494</v>
       </c>
@@ -67952,6 +67994,12 @@
       <c r="H1562" s="4" t="s">
         <v>48</v>
       </c>
+      <c r="I1562" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1562" s="4" t="s">
+        <v>1337</v>
+      </c>
       <c r="M1562" s="4" t="s">
         <v>2550</v>
       </c>
@@ -67978,6 +68026,12 @@
       <c r="H1563" s="4" t="s">
         <v>18</v>
       </c>
+      <c r="I1563" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1563" s="4" t="s">
+        <v>1337</v>
+      </c>
       <c r="M1563" s="4" t="s">
         <v>2531</v>
       </c>
@@ -68004,8 +68058,110 @@
       <c r="H1564" s="4" t="s">
         <v>948</v>
       </c>
+      <c r="I1564" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1564" s="4" t="s">
+        <v>1337</v>
+      </c>
       <c r="M1564" s="4" t="s">
         <v>2551</v>
+      </c>
+    </row>
+    <row r="1565" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1565" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1565" s="4">
+        <v>135559</v>
+      </c>
+      <c r="D1565" s="2" t="s">
+        <v>2552</v>
+      </c>
+      <c r="E1565" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1565" s="4" t="s">
+        <v>2553</v>
+      </c>
+      <c r="G1565" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1565" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I1565" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1565" s="4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="M1565" s="4" t="s">
+        <v>2498</v>
+      </c>
+    </row>
+    <row r="1566" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1566" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1566" s="4">
+        <v>144331</v>
+      </c>
+      <c r="D1566" s="2" t="s">
+        <v>2552</v>
+      </c>
+      <c r="E1566" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1566" s="4" t="s">
+        <v>2554</v>
+      </c>
+      <c r="G1566" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1566" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1566" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1566" s="4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="M1566" s="4" t="s">
+        <v>2417</v>
+      </c>
+    </row>
+    <row r="1567" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B1567" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1567" s="4">
+        <v>134281</v>
+      </c>
+      <c r="D1567" s="2" t="s">
+        <v>2552</v>
+      </c>
+      <c r="E1567" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1567" s="4" t="s">
+        <v>2555</v>
+      </c>
+      <c r="G1567" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1567" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1567" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1567" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1567" s="4" t="s">
+        <v>2418</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 18/09/2026 10:12:02,66
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1309" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90D3BC6C-9816-4BF1-9CBE-F34981014D58}"/>
+  <xr:revisionPtr revIDLastSave="1335" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17C76FF5-63F3-4483-9CFF-836CBCB01244}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$1533</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$1567</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14189" uniqueCount="2556">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14208" uniqueCount="2559">
   <si>
     <t>ID</t>
   </si>
@@ -7952,6 +7952,15 @@
   </si>
   <si>
     <t xml:space="preserve">prestador de serviço não compareceu </t>
+  </si>
+  <si>
+    <t>17/09/2026</t>
+  </si>
+  <si>
+    <t>ninguem veio fazer a manutencao programada pela 2º vez .. alegaram imprevisto / urgencia , em outro estabelecimento</t>
+  </si>
+  <si>
+    <t>nem sempre obedece um padrão, as vezes não chegam no horario combinado o que atrapalha a rotina da casa,fazem uma manutenção rapida sem explicar direito o que é feito e nos deixam um comprovante em branco,  no passado tinham mais cuidao faziam higienização interna e externa com mais cuidado.</t>
   </si>
 </sst>
 </file>
@@ -8407,7 +8416,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1567"/>
+  <dimension ref="A1:M1569"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -62181,6 +62190,9 @@
       <c r="A1408" s="4">
         <v>412</v>
       </c>
+      <c r="B1408" s="4" t="s">
+        <v>1315</v>
+      </c>
       <c r="C1408" s="4">
         <v>92325</v>
       </c>
@@ -67653,6 +67665,9 @@
       </c>
     </row>
     <row r="1552" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1552" s="4">
+        <v>573</v>
+      </c>
       <c r="B1552" s="4" t="s">
         <v>1227</v>
       </c>
@@ -67684,7 +67699,10 @@
         <v>2415</v>
       </c>
     </row>
-    <row r="1553" spans="2:13" ht="90" x14ac:dyDescent="0.25">
+    <row r="1553" spans="1:13" ht="90" x14ac:dyDescent="0.25">
+      <c r="A1553" s="4">
+        <v>574</v>
+      </c>
       <c r="B1553" s="4" t="s">
         <v>1227</v>
       </c>
@@ -67716,7 +67734,10 @@
         <v>2416</v>
       </c>
     </row>
-    <row r="1554" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="1554" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1554" s="4">
+        <v>575</v>
+      </c>
       <c r="B1554" s="4" t="s">
         <v>1315</v>
       </c>
@@ -67748,7 +67769,10 @@
         <v>2417</v>
       </c>
     </row>
-    <row r="1555" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="1555" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1555" s="4">
+        <v>576</v>
+      </c>
       <c r="B1555" s="4" t="s">
         <v>1315</v>
       </c>
@@ -67780,7 +67804,10 @@
         <v>2418</v>
       </c>
     </row>
-    <row r="1556" spans="2:13" ht="120" x14ac:dyDescent="0.25">
+    <row r="1556" spans="1:13" ht="120" x14ac:dyDescent="0.25">
+      <c r="A1556" s="4">
+        <v>577</v>
+      </c>
       <c r="B1556" s="4" t="s">
         <v>1315</v>
       </c>
@@ -67812,7 +67839,10 @@
         <v>2419</v>
       </c>
     </row>
-    <row r="1557" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="1557" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1557" s="4">
+        <v>578</v>
+      </c>
       <c r="B1557" s="4" t="s">
         <v>1227</v>
       </c>
@@ -67844,7 +67874,10 @@
         <v>2419</v>
       </c>
     </row>
-    <row r="1558" spans="2:13" ht="60" x14ac:dyDescent="0.25">
+    <row r="1558" spans="1:13" ht="60" x14ac:dyDescent="0.25">
+      <c r="A1558" s="4">
+        <v>579</v>
+      </c>
       <c r="B1558" s="4" t="s">
         <v>1315</v>
       </c>
@@ -67876,7 +67909,10 @@
         <v>2418</v>
       </c>
     </row>
-    <row r="1559" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="1559" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1559" s="4">
+        <v>580</v>
+      </c>
       <c r="B1559" s="4" t="s">
         <v>1227</v>
       </c>
@@ -67908,7 +67944,10 @@
         <v>2494</v>
       </c>
     </row>
-    <row r="1560" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="1560" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1560" s="4">
+        <v>581</v>
+      </c>
       <c r="B1560" s="4" t="s">
         <v>49</v>
       </c>
@@ -67940,7 +67979,10 @@
         <v>2453</v>
       </c>
     </row>
-    <row r="1561" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="1561" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1561" s="4">
+        <v>582</v>
+      </c>
       <c r="B1561" s="4" t="s">
         <v>1315</v>
       </c>
@@ -67972,7 +68014,10 @@
         <v>2494</v>
       </c>
     </row>
-    <row r="1562" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="1562" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1562" s="4">
+        <v>583</v>
+      </c>
       <c r="B1562" s="4" t="s">
         <v>1315</v>
       </c>
@@ -68004,7 +68049,10 @@
         <v>2550</v>
       </c>
     </row>
-    <row r="1563" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="1563" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1563" s="4">
+        <v>584</v>
+      </c>
       <c r="B1563" s="4" t="s">
         <v>49</v>
       </c>
@@ -68036,7 +68084,10 @@
         <v>2531</v>
       </c>
     </row>
-    <row r="1564" spans="2:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="1564" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1564" s="4">
+        <v>585</v>
+      </c>
       <c r="B1564" s="4" t="s">
         <v>1315</v>
       </c>
@@ -68068,7 +68119,10 @@
         <v>2551</v>
       </c>
     </row>
-    <row r="1565" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="1565" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1565" s="4">
+        <v>586</v>
+      </c>
       <c r="B1565" s="4" t="s">
         <v>1227</v>
       </c>
@@ -68100,7 +68154,10 @@
         <v>2498</v>
       </c>
     </row>
-    <row r="1566" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="1566" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1566" s="4">
+        <v>587</v>
+      </c>
       <c r="B1566" s="4" t="s">
         <v>1227</v>
       </c>
@@ -68132,7 +68189,10 @@
         <v>2417</v>
       </c>
     </row>
-    <row r="1567" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="1567" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1567" s="4">
+        <v>588</v>
+      </c>
       <c r="B1567" s="4" t="s">
         <v>1315</v>
       </c>
@@ -68162,6 +68222,76 @@
       </c>
       <c r="M1567" s="4" t="s">
         <v>2418</v>
+      </c>
+    </row>
+    <row r="1568" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1568" s="4">
+        <v>589</v>
+      </c>
+      <c r="B1568" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1568" s="4">
+        <v>126474</v>
+      </c>
+      <c r="D1568" s="2" t="s">
+        <v>2556</v>
+      </c>
+      <c r="E1568" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1568" s="4" t="s">
+        <v>2557</v>
+      </c>
+      <c r="G1568" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1568" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1568" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1568" s="4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="M1568" s="4" t="s">
+        <v>2512</v>
+      </c>
+    </row>
+    <row r="1569" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1569" s="4">
+        <v>590</v>
+      </c>
+      <c r="B1569" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1569" s="4">
+        <v>139100</v>
+      </c>
+      <c r="D1569" s="2" t="s">
+        <v>2556</v>
+      </c>
+      <c r="E1569" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1569" s="4" t="s">
+        <v>2558</v>
+      </c>
+      <c r="G1569" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1569" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I1569" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1569" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1569" s="4" t="s">
+        <v>2534</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 21/09/2026 11:11:46,30
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1335" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17C76FF5-63F3-4483-9CFF-836CBCB01244}"/>
+  <xr:revisionPtr revIDLastSave="1344" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1A6D2A3-4B63-458B-BF11-C63F69D3457A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14208" uniqueCount="2559">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14217" uniqueCount="2561">
   <si>
     <t>ID</t>
   </si>
@@ -7961,6 +7961,12 @@
   </si>
   <si>
     <t>nem sempre obedece um padrão, as vezes não chegam no horario combinado o que atrapalha a rotina da casa,fazem uma manutenção rapida sem explicar direito o que é feito e nos deixam um comprovante em branco,  no passado tinham mais cuidao faziam higienização interna e externa com mais cuidado.</t>
+  </si>
+  <si>
+    <t>18/09/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Porque nao me notificaram via WhatsApp que estava com 2 pagamentos em atraso. Troquei o cartão por perda . Trocaram meu purificador e deixaram vazando até hoje e qdo fui pedir o retorno do técnico foi qdo descobri o atraso de pagamentos e que so podia solicitar seevicos após a quitacao. Me mandaram um boleto que nao abre com meu cpf . Logo não consigo pagar e nem beber água filtrada sem falar no vazamento na cozinha . </t>
   </si>
 </sst>
 </file>
@@ -8416,7 +8422,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1569"/>
+  <dimension ref="A1:M1570"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -68294,6 +68300,41 @@
         <v>2534</v>
       </c>
     </row>
+    <row r="1570" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1570" s="4">
+        <v>591</v>
+      </c>
+      <c r="B1570" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1570" s="4">
+        <v>130568</v>
+      </c>
+      <c r="D1570" s="2" t="s">
+        <v>2559</v>
+      </c>
+      <c r="E1570" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1570" s="4" t="s">
+        <v>2560</v>
+      </c>
+      <c r="G1570" s="4" t="s">
+        <v>1418</v>
+      </c>
+      <c r="H1570" s="4" t="s">
+        <v>1443</v>
+      </c>
+      <c r="I1570" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1570" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1570" s="4" t="s">
+        <v>2494</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 22/09/2026 10:49:17,83
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1344" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1A6D2A3-4B63-458B-BF11-C63F69D3457A}"/>
+  <xr:revisionPtr revIDLastSave="1476" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70A0C2CF-C829-4045-9B72-C4AD9323F3C8}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$1567</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$1570</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14217" uniqueCount="2561">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14281" uniqueCount="2570">
   <si>
     <t>ID</t>
   </si>
@@ -7967,6 +7967,34 @@
   </si>
   <si>
     <t xml:space="preserve">Porque nao me notificaram via WhatsApp que estava com 2 pagamentos em atraso. Troquei o cartão por perda . Trocaram meu purificador e deixaram vazando até hoje e qdo fui pedir o retorno do técnico foi qdo descobri o atraso de pagamentos e que so podia solicitar seevicos após a quitacao. Me mandaram um boleto que nao abre com meu cpf . Logo não consigo pagar e nem beber água filtrada sem falar no vazamento na cozinha . </t>
+  </si>
+  <si>
+    <t>21/09/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Só tivemos 1 manutenção até agora. Ano passado </t>
+  </si>
+  <si>
+    <t>Falta de pessoalidade e situações que não acontecem...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eu estava no processo de mudança tudo muito corrido e técnico veio instalar o purificador no meu novo endereço porém ele instalou o purificador em um local impróprio que está atrapalhando toda a logística da casa , e na hora não observei pois eu estava no corre corre da mudança. </t>
+  </si>
+  <si>
+    <t>Depois que foi transferido para a Culligan o serviço ficou pessimo. Minha manutenção estava, primeiramente, angendada para o dia 03/09 e não apareceu ninguem. Foi reagendada para 15/09 e também o tecnico não compareceu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Existe muita demora no atendimento presencial dos técnicos. </t>
+  </si>
+  <si>
+    <t>02 visitas técnicas sem nenhuma solução.</t>
+  </si>
+  <si>
+    <t>Pessimo!!!! Marcaram 3 vez e nao vieram</t>
+  </si>
+  <si>
+    <t>Sem compromissos nas visitas agendadas.
+Não cumprem as datas.</t>
   </si>
 </sst>
 </file>
@@ -8422,7 +8450,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1570"/>
+  <dimension ref="A1:M1578"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -67164,10 +67192,10 @@
         <v>1654</v>
       </c>
       <c r="G1538" s="4" t="s">
-        <v>15</v>
+        <v>65</v>
       </c>
       <c r="H1538" s="4" t="s">
-        <v>40</v>
+        <v>1435</v>
       </c>
       <c r="I1538" s="4" t="s">
         <v>1308</v>
@@ -68333,6 +68361,262 @@
       </c>
       <c r="M1570" s="4" t="s">
         <v>2494</v>
+      </c>
+    </row>
+    <row r="1571" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1571" s="4">
+        <v>592</v>
+      </c>
+      <c r="B1571" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1571" s="4">
+        <v>133394</v>
+      </c>
+      <c r="D1571" s="2" t="s">
+        <v>2561</v>
+      </c>
+      <c r="E1571" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1571" s="4" t="s">
+        <v>2562</v>
+      </c>
+      <c r="G1571" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1571" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="J1571" s="4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="M1571" s="4" t="s">
+        <v>2494</v>
+      </c>
+    </row>
+    <row r="1572" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1572" s="4">
+        <v>593</v>
+      </c>
+      <c r="B1572" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1572" s="4">
+        <v>141810</v>
+      </c>
+      <c r="D1572" s="2" t="s">
+        <v>2561</v>
+      </c>
+      <c r="E1572" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1572" s="4" t="s">
+        <v>2563</v>
+      </c>
+      <c r="G1572" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1572" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J1572" s="4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="M1572" s="4" t="s">
+        <v>2540</v>
+      </c>
+    </row>
+    <row r="1573" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1573" s="4">
+        <v>594</v>
+      </c>
+      <c r="B1573" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1573" s="4">
+        <v>146746</v>
+      </c>
+      <c r="D1573" s="2" t="s">
+        <v>2561</v>
+      </c>
+      <c r="E1573" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1573" s="4" t="s">
+        <v>2564</v>
+      </c>
+      <c r="G1573" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1573" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="J1573" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1573" s="4" t="s">
+        <v>2501</v>
+      </c>
+    </row>
+    <row r="1574" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1574" s="4">
+        <v>595</v>
+      </c>
+      <c r="B1574" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1574" s="4">
+        <v>139315</v>
+      </c>
+      <c r="D1574" s="2" t="s">
+        <v>2561</v>
+      </c>
+      <c r="E1574" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1574" s="4" t="s">
+        <v>2565</v>
+      </c>
+      <c r="G1574" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1574" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="J1574" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1574" s="4" t="s">
+        <v>2418</v>
+      </c>
+    </row>
+    <row r="1575" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1575" s="4">
+        <v>596</v>
+      </c>
+      <c r="B1575" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1575" s="4">
+        <v>140718</v>
+      </c>
+      <c r="D1575" s="2" t="s">
+        <v>2561</v>
+      </c>
+      <c r="E1575" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1575" s="4" t="s">
+        <v>2566</v>
+      </c>
+      <c r="G1575" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1575" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1575" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1575" s="4" t="s">
+        <v>2498</v>
+      </c>
+    </row>
+    <row r="1576" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1576" s="4">
+        <v>597</v>
+      </c>
+      <c r="B1576" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1576" s="4">
+        <v>145518</v>
+      </c>
+      <c r="D1576" s="2" t="s">
+        <v>2561</v>
+      </c>
+      <c r="E1576" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1576" s="4" t="s">
+        <v>2567</v>
+      </c>
+      <c r="G1576" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1576" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1576" s="4" t="s">
+        <v>1339</v>
+      </c>
+      <c r="M1576" s="4" t="s">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="1577" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1577" s="4">
+        <v>598</v>
+      </c>
+      <c r="B1577" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1577" s="4">
+        <v>146533</v>
+      </c>
+      <c r="D1577" s="2" t="s">
+        <v>2561</v>
+      </c>
+      <c r="E1577" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1577" s="4" t="s">
+        <v>2568</v>
+      </c>
+      <c r="G1577" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1577" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="J1577" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1577" s="4" t="s">
+        <v>2416</v>
+      </c>
+    </row>
+    <row r="1578" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1578" s="4">
+        <v>599</v>
+      </c>
+      <c r="B1578" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1578" s="4">
+        <v>135603</v>
+      </c>
+      <c r="D1578" s="2" t="s">
+        <v>2561</v>
+      </c>
+      <c r="E1578" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1578" s="5" t="s">
+        <v>2569</v>
+      </c>
+      <c r="G1578" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1578" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="J1578" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1578" s="4" t="s">
+        <v>2531</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 23/09/2026  9:46:05,38
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1476" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70A0C2CF-C829-4045-9B72-C4AD9323F3C8}"/>
+  <xr:revisionPtr revIDLastSave="1491" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{68BCEA38-1491-48A7-966E-0733E5EEA57F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14281" uniqueCount="2570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14307" uniqueCount="2573">
   <si>
     <t>ID</t>
   </si>
@@ -7995,6 +7995,15 @@
   <si>
     <t>Sem compromissos nas visitas agendadas.
 Não cumprem as datas.</t>
+  </si>
+  <si>
+    <t>22/09/2026</t>
+  </si>
+  <si>
+    <t>DEMOROU 2 MESES PARA SER EFETUADA A TROCA DO FILTRO QUE JA PAROU DE FUNCIONAR 3X E QUANDO O TECNICO VEIO FAZER A TROCA O FILTRO  QUE DEVERIA SER NOVO QUEBRADO. MAS ELE SÓ VIU APÓS INSTALAR. COMO MEU FILTRO ANTIGO FICA SOBRE UM SUPORTE DE PAREDE ELE RECOLOCOU ENTÃO O FILTRO ANTIGO SEM O PREDER, DE QUALQUER JEITO E TODO TORTO CORRENDO O RISCO DE QUEDA. FICOU DE VOLTAR AQUI NO DIA SEGUINTE COM OUTRO FILTRO E NÃO VEIO. ESTOU BEM INSATISFEITA E NÃO ACEITO TEREM LARGADO MEU FILTRO ANTIGO DESSA MANEIRA, PODENDO CAUSAR UM ACIDENTE.</t>
+  </si>
+  <si>
+    <t>Pela dificuldade que tive na solução do problema. Se têm acesso ao histórico poderão verificar. O problema do meu aparelho foi solucionado, mas em seguida notei um superaquecimento na parte superior. Não consegui falar para tentar uma solução. Estou com receio de mantê-lo ligado e causar um dano maior. Nada a reclamar do atendimento técnico.</t>
   </si>
 </sst>
 </file>
@@ -8450,7 +8459,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1578"/>
+  <dimension ref="A1:M1580"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -68388,6 +68397,9 @@
       <c r="H1571" s="4" t="s">
         <v>948</v>
       </c>
+      <c r="I1571" s="4" t="s">
+        <v>1308</v>
+      </c>
       <c r="J1571" s="4" t="s">
         <v>1338</v>
       </c>
@@ -68420,6 +68432,9 @@
       <c r="H1572" s="4" t="s">
         <v>21</v>
       </c>
+      <c r="I1572" s="4" t="s">
+        <v>1308</v>
+      </c>
       <c r="J1572" s="4" t="s">
         <v>1338</v>
       </c>
@@ -68452,6 +68467,9 @@
       <c r="H1573" s="4" t="s">
         <v>40</v>
       </c>
+      <c r="I1573" s="4" t="s">
+        <v>1308</v>
+      </c>
       <c r="J1573" s="4" t="s">
         <v>1337</v>
       </c>
@@ -68484,6 +68502,9 @@
       <c r="H1574" s="4" t="s">
         <v>948</v>
       </c>
+      <c r="I1574" s="4" t="s">
+        <v>1308</v>
+      </c>
       <c r="J1574" s="4" t="s">
         <v>1337</v>
       </c>
@@ -68516,6 +68537,9 @@
       <c r="H1575" s="4" t="s">
         <v>26</v>
       </c>
+      <c r="I1575" s="4" t="s">
+        <v>1308</v>
+      </c>
       <c r="J1575" s="4" t="s">
         <v>1337</v>
       </c>
@@ -68548,6 +68572,9 @@
       <c r="H1576" s="4" t="s">
         <v>18</v>
       </c>
+      <c r="I1576" s="4" t="s">
+        <v>1308</v>
+      </c>
       <c r="J1576" s="4" t="s">
         <v>1339</v>
       </c>
@@ -68580,6 +68607,9 @@
       <c r="H1577" s="4" t="s">
         <v>948</v>
       </c>
+      <c r="I1577" s="4" t="s">
+        <v>1308</v>
+      </c>
       <c r="J1577" s="4" t="s">
         <v>1337</v>
       </c>
@@ -68612,11 +68642,84 @@
       <c r="H1578" s="4" t="s">
         <v>948</v>
       </c>
+      <c r="I1578" s="4" t="s">
+        <v>1308</v>
+      </c>
       <c r="J1578" s="4" t="s">
         <v>1337</v>
       </c>
       <c r="M1578" s="4" t="s">
         <v>2531</v>
+      </c>
+    </row>
+    <row r="1579" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1579" s="4">
+        <v>600</v>
+      </c>
+      <c r="B1579" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1579" s="4">
+        <v>146697</v>
+      </c>
+      <c r="D1579" s="2" t="s">
+        <v>2570</v>
+      </c>
+      <c r="E1579" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1579" s="4" t="s">
+        <v>2571</v>
+      </c>
+      <c r="G1579" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1579" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I1579" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1579" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1579" s="4" t="s">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="1580" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1580" s="4">
+        <v>601</v>
+      </c>
+      <c r="B1580" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1580" s="4">
+        <v>147829</v>
+      </c>
+      <c r="D1580" s="2" t="s">
+        <v>2570</v>
+      </c>
+      <c r="E1580" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1580" s="4" t="s">
+        <v>2572</v>
+      </c>
+      <c r="G1580" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1580" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1580" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1580" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1580" s="4" t="s">
+        <v>2490</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 24/09/2026 10:57:24,04
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1491" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{68BCEA38-1491-48A7-966E-0733E5EEA57F}"/>
+  <xr:revisionPtr revIDLastSave="1501" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A1709E1-82E1-4715-9E0A-003860678BBE}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$1570</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14307" uniqueCount="2573">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14334" uniqueCount="2578">
   <si>
     <t>ID</t>
   </si>
@@ -8004,6 +8004,23 @@
   </si>
   <si>
     <t>Pela dificuldade que tive na solução do problema. Se têm acesso ao histórico poderão verificar. O problema do meu aparelho foi solucionado, mas em seguida notei um superaquecimento na parte superior. Não consegui falar para tentar uma solução. Estou com receio de mantê-lo ligado e causar um dano maior. Nada a reclamar do atendimento técnico.</t>
+  </si>
+  <si>
+    <t>23/09/2026</t>
+  </si>
+  <si>
+    <t>24/09/2026</t>
+  </si>
+  <si>
+    <t>O atendimento dos técnicos é sempre muito bom, porém o atendimento ao cliente deixa a desejar, sou cliente ha 20 ou mais anos e no mês de Agosto tive pedido de troca de elemento filtrante negado devido a uma fatura do mês de Abril acredito,nunca fui cobrado , so soube quando liguei para pedir a substituição do elemento filtrante,  um total descaso com um cliente antigo,  não vou dar um golpe de uma mensalidade na Brastemp ! E a resposta será que o sistema não permite! Ridiculo!!</t>
+  </si>
+  <si>
+    <t>O técnico mudou o purificador antes da data combinada gerando transtornos para minha família. Adicionalmente, não instalou o suporte de parede como solicitei. Em outras palavras, fez o que deu na telha.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FOI FEITO MANUTENÇÃO PERIODICA DOS BEBEDOUROS DE AGUA, DIA 18/09/26, APOS ESTA MANUTENÇÃO FICOU SAINDO POUCA  AGUA E NÃO GELANDO. FIZ UM NOVO CHAMADO QUE SERIA DIA 24/09 NO PERIODO DA TARDE, MAS NO DIA 23/09 PELA MANHA VEIO UM TECNICO CHAMADO BRUNO, PEDIMOS A SENHA, ELE NÃO SOUBE INFORMAR E AINDA FOI MUITO MAL EDUCADO COM A GENTE, DIZENDO QUE ENTÃO IRIA EMBORA, ENTÃO FALAMOS PARA ELE IR EMBORA, QUESTÃO DE SEGURANÇA. DEPOIS ENTREI EM CONTATO COM O ATENDIMENTO E TIVE QUE CANCELAR A VISITA DO DIA 24/09, POIS A ATENTENDE NAIRA NÃO TINHA CADASTRADO A SENHA, AGORA VOU TER QUE ENTRAR NOVAMENTE EM CONTATO, PARA AGENDAR UMA NOVO VISITA.
+RESUMINDO FUNCIONARIOS OU TERCEIRIZADOS DESPREPARADOS,
+</t>
   </si>
 </sst>
 </file>
@@ -8459,7 +8476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1580"/>
+  <dimension ref="A1:M1583"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -68722,6 +68739,102 @@
         <v>2490</v>
       </c>
     </row>
+    <row r="1581" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B1581" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1581" s="4">
+        <v>146253</v>
+      </c>
+      <c r="D1581" s="2" t="s">
+        <v>2573</v>
+      </c>
+      <c r="E1581" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1581" s="4" t="s">
+        <v>2575</v>
+      </c>
+      <c r="G1581" s="4" t="s">
+        <v>1418</v>
+      </c>
+      <c r="H1581" s="4" t="s">
+        <v>1443</v>
+      </c>
+      <c r="I1581" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1581" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1581" s="4" t="s">
+        <v>2419</v>
+      </c>
+    </row>
+    <row r="1582" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B1582" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1582" s="4">
+        <v>147565</v>
+      </c>
+      <c r="D1582" s="2" t="s">
+        <v>2573</v>
+      </c>
+      <c r="E1582" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1582" s="4" t="s">
+        <v>2576</v>
+      </c>
+      <c r="G1582" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1582" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I1582" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1582" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1582" s="4" t="s">
+        <v>2452</v>
+      </c>
+    </row>
+    <row r="1583" spans="1:13" ht="270" x14ac:dyDescent="0.25">
+      <c r="B1583" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1583" s="4">
+        <v>146447</v>
+      </c>
+      <c r="D1583" s="2" t="s">
+        <v>2574</v>
+      </c>
+      <c r="E1583" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1583" s="5" t="s">
+        <v>2577</v>
+      </c>
+      <c r="G1583" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1583" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1583" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1583" s="4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="M1583" s="4" t="s">
+        <v>2517</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 25/09/2026 10:07:30,82
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1501" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A1709E1-82E1-4715-9E0A-003860678BBE}"/>
+  <xr:revisionPtr revIDLastSave="1518" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF8FCEF0-86EA-45D3-947B-B74BDF9E5ECC}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$1570</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14334" uniqueCount="2578">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14370" uniqueCount="2584">
   <si>
     <t>ID</t>
   </si>
@@ -8021,6 +8021,24 @@
     <t xml:space="preserve">FOI FEITO MANUTENÇÃO PERIODICA DOS BEBEDOUROS DE AGUA, DIA 18/09/26, APOS ESTA MANUTENÇÃO FICOU SAINDO POUCA  AGUA E NÃO GELANDO. FIZ UM NOVO CHAMADO QUE SERIA DIA 24/09 NO PERIODO DA TARDE, MAS NO DIA 23/09 PELA MANHA VEIO UM TECNICO CHAMADO BRUNO, PEDIMOS A SENHA, ELE NÃO SOUBE INFORMAR E AINDA FOI MUITO MAL EDUCADO COM A GENTE, DIZENDO QUE ENTÃO IRIA EMBORA, ENTÃO FALAMOS PARA ELE IR EMBORA, QUESTÃO DE SEGURANÇA. DEPOIS ENTREI EM CONTATO COM O ATENDIMENTO E TIVE QUE CANCELAR A VISITA DO DIA 24/09, POIS A ATENTENDE NAIRA NÃO TINHA CADASTRADO A SENHA, AGORA VOU TER QUE ENTRAR NOVAMENTE EM CONTATO, PARA AGENDAR UMA NOVO VISITA.
 RESUMINDO FUNCIONARIOS OU TERCEIRIZADOS DESPREPARADOS,
 </t>
+  </si>
+  <si>
+    <t>O preço pago mensalmente é inviável, em um ano dar pra comprar um bom filtro, sem pagar mensalidade. Pensando seriamente em cancelar …</t>
+  </si>
+  <si>
+    <t>Extrema morosidade no atendimento referente a instalação de novos filtros.</t>
+  </si>
+  <si>
+    <t>Péssimo atendimento, so via telefone pra agendar visita tecnica, marcam um dia e depois mandam um e-mail com outra data nada a ver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pq me faz perder meio dia para aguardar a chegada do técnico.  Esse agendamento tem de ser em um intervalo menor, talvez de 2 em 2 horas para não fazer o cliente ficar a disposição da visita , e avaliar a troca do aparelho por um concorrente que não o faça perder tanto tempo </t>
+  </si>
+  <si>
+    <t>25/09/2026</t>
+  </si>
+  <si>
+    <t>Aquisição</t>
   </si>
 </sst>
 </file>
@@ -8476,7 +8494,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1583"/>
+  <dimension ref="A1:M1587"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -68740,6 +68758,9 @@
       </c>
     </row>
     <row r="1581" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1581" s="4">
+        <v>602</v>
+      </c>
       <c r="B1581" s="4" t="s">
         <v>1227</v>
       </c>
@@ -68772,6 +68793,9 @@
       </c>
     </row>
     <row r="1582" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1582" s="4">
+        <v>603</v>
+      </c>
       <c r="B1582" s="4" t="s">
         <v>1227</v>
       </c>
@@ -68804,6 +68828,9 @@
       </c>
     </row>
     <row r="1583" spans="1:13" ht="270" x14ac:dyDescent="0.25">
+      <c r="A1583" s="4">
+        <v>604</v>
+      </c>
       <c r="B1583" s="4" t="s">
         <v>1315</v>
       </c>
@@ -68833,6 +68860,146 @@
       </c>
       <c r="M1583" s="4" t="s">
         <v>2517</v>
+      </c>
+    </row>
+    <row r="1584" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1584" s="4">
+        <v>605</v>
+      </c>
+      <c r="B1584" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1584" s="4">
+        <v>147640</v>
+      </c>
+      <c r="D1584" s="2" t="s">
+        <v>2574</v>
+      </c>
+      <c r="E1584" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1584" s="4" t="s">
+        <v>2578</v>
+      </c>
+      <c r="G1584" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1584" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="I1584" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1584" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1584" s="4" t="s">
+        <v>2452</v>
+      </c>
+    </row>
+    <row r="1585" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1585" s="4">
+        <v>606</v>
+      </c>
+      <c r="B1585" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1585" s="4">
+        <v>134800</v>
+      </c>
+      <c r="D1585" s="2" t="s">
+        <v>2574</v>
+      </c>
+      <c r="E1585" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1585" s="4" t="s">
+        <v>2579</v>
+      </c>
+      <c r="G1585" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="H1585" s="4" t="s">
+        <v>2583</v>
+      </c>
+      <c r="I1585" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1585" s="4" t="s">
+        <v>1359</v>
+      </c>
+      <c r="M1585" s="4" t="s">
+        <v>2491</v>
+      </c>
+    </row>
+    <row r="1586" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1586" s="4">
+        <v>607</v>
+      </c>
+      <c r="B1586" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1586" s="4">
+        <v>149594</v>
+      </c>
+      <c r="D1586" s="2" t="s">
+        <v>2574</v>
+      </c>
+      <c r="E1586" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1586" s="4" t="s">
+        <v>2580</v>
+      </c>
+      <c r="G1586" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1586" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="I1586" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1586" s="4" t="s">
+        <v>1339</v>
+      </c>
+      <c r="M1586" s="4" t="s">
+        <v>2502</v>
+      </c>
+    </row>
+    <row r="1587" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1587" s="4">
+        <v>608</v>
+      </c>
+      <c r="B1587" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1587" s="4">
+        <v>139831</v>
+      </c>
+      <c r="D1587" s="2" t="s">
+        <v>2582</v>
+      </c>
+      <c r="E1587" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1587" s="4" t="s">
+        <v>2581</v>
+      </c>
+      <c r="G1587" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1587" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1587" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1587" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1587" s="4" t="s">
+        <v>2452</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 28/09/2026  9:58:40,01
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1518" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF8FCEF0-86EA-45D3-947B-B74BDF9E5ECC}"/>
+  <xr:revisionPtr revIDLastSave="1535" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D11FE8E7-6BEA-451C-9552-DACDBDE73AF2}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14370" uniqueCount="2584">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14415" uniqueCount="2591">
   <si>
     <t>ID</t>
   </si>
@@ -8039,6 +8039,29 @@
   </si>
   <si>
     <t>Aquisição</t>
+  </si>
+  <si>
+    <t>26/09/2026</t>
+  </si>
+  <si>
+    <t>28/09/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Instalação com aspecto de favela, área que nenhuma pessoa gostaria ou deveria viver mas que a realidade impõe infelizmente às pessoas menos favorecidas. 
+Pedido ao instalador para modificar, disse que não faria. Como não assinamos a OS, se foi assinada, não é nossa assinatura. 
+Péssimo, deplorável. Jamais recomendável. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demora de 20 dias para primeira data de agendamento, culligan faltou e nao deu satisfação. Tentei atendimento e fiquei sem nenhuma resposta. Vcs tem 3 meses u 4 WhatsApp automatizados q funcionam muito mal e sem opção de atendente. Finalmente vcs entraram em contato p nova data sem nem pedir desculpas. Péssima experiência, mas produto é bom e por isso mantive contrato. Mas ja estou preocupado quando precisar de algum serviço </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não recebi nem manutenção esse mês </t>
+  </si>
+  <si>
+    <t>Os instaladores necessitam ( com urgência) passar por reciclagem sobre atendimento ao cliente</t>
+  </si>
+  <si>
+    <t>Desorganização para atendimento remoto. Sem pós venda não tem como manter qualidade</t>
   </si>
 </sst>
 </file>
@@ -8494,7 +8517,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1587"/>
+  <dimension ref="A1:M1592"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -8507,8 +8530,8 @@
     <col min="8" max="8" width="28" style="4" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15.5703125" style="4" customWidth="1"/>
     <col min="10" max="10" width="18.140625" style="4" customWidth="1"/>
-    <col min="11" max="11" width="30" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.5703125" style="4" customWidth="1"/>
+    <col min="11" max="11" width="30" style="4" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="8.5703125" style="4" hidden="1" customWidth="1"/>
     <col min="13" max="13" width="36.28515625" style="4" bestFit="1" customWidth="1"/>
     <col min="14" max="16384" width="9.140625" style="4"/>
   </cols>
@@ -69002,6 +69025,181 @@
         <v>2452</v>
       </c>
     </row>
+    <row r="1588" spans="1:13" ht="105" x14ac:dyDescent="0.25">
+      <c r="A1588" s="4">
+        <v>609</v>
+      </c>
+      <c r="B1588" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1588" s="4">
+        <v>143048</v>
+      </c>
+      <c r="D1588" s="2" t="s">
+        <v>2582</v>
+      </c>
+      <c r="E1588" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1588" s="5" t="s">
+        <v>2586</v>
+      </c>
+      <c r="G1588" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1588" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I1588" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1588" s="4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="M1588" s="4" t="s">
+        <v>2490</v>
+      </c>
+    </row>
+    <row r="1589" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1589" s="4">
+        <v>610</v>
+      </c>
+      <c r="B1589" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1589" s="4">
+        <v>148758</v>
+      </c>
+      <c r="D1589" s="2" t="s">
+        <v>2582</v>
+      </c>
+      <c r="E1589" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1589" s="4" t="s">
+        <v>2587</v>
+      </c>
+      <c r="G1589" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="H1589" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="I1589" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1589" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1589" s="4" t="s">
+        <v>2528</v>
+      </c>
+    </row>
+    <row r="1590" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1590" s="4">
+        <v>611</v>
+      </c>
+      <c r="B1590" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1590" s="4">
+        <v>149512</v>
+      </c>
+      <c r="D1590" s="2" t="s">
+        <v>2584</v>
+      </c>
+      <c r="E1590" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1590" s="4" t="s">
+        <v>2588</v>
+      </c>
+      <c r="G1590" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1590" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1590" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1590" s="4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="M1590" s="4" t="s">
+        <v>2452</v>
+      </c>
+    </row>
+    <row r="1591" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1591" s="4">
+        <v>612</v>
+      </c>
+      <c r="B1591" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1591" s="4">
+        <v>143798</v>
+      </c>
+      <c r="D1591" s="2" t="s">
+        <v>2584</v>
+      </c>
+      <c r="E1591" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1591" s="4" t="s">
+        <v>2589</v>
+      </c>
+      <c r="G1591" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1591" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I1591" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1591" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1591" s="4" t="s">
+        <v>2499</v>
+      </c>
+    </row>
+    <row r="1592" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1592" s="4">
+        <v>613</v>
+      </c>
+      <c r="B1592" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1592" s="4">
+        <v>149689</v>
+      </c>
+      <c r="D1592" s="2" t="s">
+        <v>2585</v>
+      </c>
+      <c r="E1592" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1592" s="4" t="s">
+        <v>2590</v>
+      </c>
+      <c r="G1592" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1592" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="I1592" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1592" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1592" s="4" t="s">
+        <v>2494</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 29/09/2026  9:14:54,57
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1535" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D11FE8E7-6BEA-451C-9552-DACDBDE73AF2}"/>
+  <xr:revisionPtr revIDLastSave="1554" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{699D063B-C65E-480A-80A8-D85194123DB8}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14415" uniqueCount="2591">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14460" uniqueCount="2597">
   <si>
     <t>ID</t>
   </si>
@@ -8062,6 +8062,25 @@
   </si>
   <si>
     <t>Desorganização para atendimento remoto. Sem pós venda não tem como manter qualidade</t>
+  </si>
+  <si>
+    <t>29/09/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tenho um contrato com filtro de agua em debito automatico! pararam as cobranças eu liguei varias vezes mais sem resultado. agora vcs resolvem cobrar tudo de 1 só vez e pior fiquei meses sem manutenção da onde vem isso???
+</t>
+  </si>
+  <si>
+    <t>Demora no atendimento, e demora para responder os e-mails</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fiquei muito tempo com filtro parado por falta de técnicos na minha região . Agora , após a troca do filtro, gostaria de começar a pagar novamente mas não consigo nenhum contato com a Brastemp. Tudo robotizado. </t>
+  </si>
+  <si>
+    <t>Pela segunda vez o técnico não apareceu!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estou aguadando a troca do aparelho , e nada ,já estou sem agua gelada a 20 ou mais </t>
   </si>
 </sst>
 </file>
@@ -8517,7 +8536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1592"/>
+  <dimension ref="A1:M1597"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -69200,6 +69219,181 @@
         <v>2494</v>
       </c>
     </row>
+    <row r="1593" spans="1:13" ht="90" x14ac:dyDescent="0.25">
+      <c r="A1593" s="4">
+        <v>614</v>
+      </c>
+      <c r="B1593" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1593" s="4">
+        <v>143265</v>
+      </c>
+      <c r="D1593" s="2" t="s">
+        <v>2585</v>
+      </c>
+      <c r="E1593" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1593" s="5" t="s">
+        <v>2592</v>
+      </c>
+      <c r="G1593" s="4" t="s">
+        <v>1418</v>
+      </c>
+      <c r="H1593" s="4" t="s">
+        <v>1443</v>
+      </c>
+      <c r="I1593" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1593" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1593" s="4" t="s">
+        <v>2418</v>
+      </c>
+    </row>
+    <row r="1594" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1594" s="4">
+        <v>615</v>
+      </c>
+      <c r="B1594" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1594" s="4">
+        <v>146263</v>
+      </c>
+      <c r="D1594" s="2" t="s">
+        <v>2585</v>
+      </c>
+      <c r="E1594" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1594" s="4" t="s">
+        <v>2593</v>
+      </c>
+      <c r="G1594" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1594" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1594" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1594" s="4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="M1594" s="4" t="s">
+        <v>2419</v>
+      </c>
+    </row>
+    <row r="1595" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1595" s="4">
+        <v>616</v>
+      </c>
+      <c r="B1595" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1595" s="4">
+        <v>123906</v>
+      </c>
+      <c r="D1595" s="2" t="s">
+        <v>2585</v>
+      </c>
+      <c r="E1595" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1595" s="4" t="s">
+        <v>2594</v>
+      </c>
+      <c r="G1595" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1595" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="I1595" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1595" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1595" s="4" t="s">
+        <v>2535</v>
+      </c>
+    </row>
+    <row r="1596" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1596" s="4">
+        <v>617</v>
+      </c>
+      <c r="B1596" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1596" s="4">
+        <v>152889</v>
+      </c>
+      <c r="D1596" s="2" t="s">
+        <v>2585</v>
+      </c>
+      <c r="E1596" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1596" s="4" t="s">
+        <v>2595</v>
+      </c>
+      <c r="G1596" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1596" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1596" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1596" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1596" s="4" t="s">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="1597" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1597" s="4">
+        <v>618</v>
+      </c>
+      <c r="B1597" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1597" s="4">
+        <v>146674</v>
+      </c>
+      <c r="D1597" s="2" t="s">
+        <v>2591</v>
+      </c>
+      <c r="E1597" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1597" s="4" t="s">
+        <v>2596</v>
+      </c>
+      <c r="G1597" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="H1597" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="I1597" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1597" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1597" s="4" t="s">
+        <v>2416</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 30/09/2026 10:04:37,57
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1554" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{699D063B-C65E-480A-80A8-D85194123DB8}"/>
+  <xr:revisionPtr revIDLastSave="1565" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{843F0FF0-8958-4349-836F-3761DA2EF825}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14460" uniqueCount="2597">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14468" uniqueCount="2598">
   <si>
     <t>ID</t>
   </si>
@@ -8081,6 +8081,9 @@
   </si>
   <si>
     <t xml:space="preserve">Estou aguadando a troca do aparelho , e nada ,já estou sem agua gelada a 20 ou mais </t>
+  </si>
+  <si>
+    <t>Manutenção péssima...desde o agendamento ao atendimento...</t>
   </si>
 </sst>
 </file>
@@ -8536,7 +8539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1597"/>
+  <dimension ref="A1:M1598"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -69394,6 +69397,38 @@
         <v>2416</v>
       </c>
     </row>
+    <row r="1598" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1598" s="4">
+        <v>619</v>
+      </c>
+      <c r="B1598" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1598" s="4">
+        <v>153041</v>
+      </c>
+      <c r="D1598" s="2" t="s">
+        <v>2591</v>
+      </c>
+      <c r="F1598" s="4" t="s">
+        <v>2597</v>
+      </c>
+      <c r="G1598" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1598" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1598" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1598" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1598" s="4" t="s">
+        <v>2416</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 01/10/2026  9:03:15,05
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1565" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{843F0FF0-8958-4349-836F-3761DA2EF825}"/>
+  <xr:revisionPtr revIDLastSave="1580" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{867868CF-50ED-4178-A3BB-C643B59A8292}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14468" uniqueCount="2598">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14496" uniqueCount="2602">
   <si>
     <t>ID</t>
   </si>
@@ -8084,6 +8084,19 @@
   </si>
   <si>
     <t>Manutenção péssima...desde o agendamento ao atendimento...</t>
+  </si>
+  <si>
+    <t>30/09/2026</t>
+  </si>
+  <si>
+    <t>Dificuldade no agendamento, empresa mal preparada para atender no agendamento, perderam solicitação de reparo ou troca realizada em março de 2026, desde então meu equipamento apresentando problemas. Para agenmdar agora foi muito vomplicado e difícil,poucas datas e desprepara nos atendentes. Estou seriamente disposto a cancelar meinha assinatura.</t>
+  </si>
+  <si>
+    <t>Durante o processo de vendas uma das perguntas que fiz expressamente é se todas as ferragens necessárias para a fixação em parede estariam incluídas na instalação e a resposta fio que sim. 
+No dia marcado para a instalação, que seria entre 8h e 13h. O instalador apareceu aos 48 do segundo tempo (13h10 aproximadamente) e informou que a Brastemp NÃO fornece/tem suporte para fixar em parede o filtro adquirido.</t>
+  </si>
+  <si>
+    <t>O serviço de agendamento e suporte ao cliente é muito problemático.</t>
   </si>
 </sst>
 </file>
@@ -8539,7 +8552,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1598"/>
+  <dimension ref="A1:M1601"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -69410,6 +69423,9 @@
       <c r="D1598" s="2" t="s">
         <v>2591</v>
       </c>
+      <c r="E1598" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="F1598" s="4" t="s">
         <v>2597</v>
       </c>
@@ -69427,6 +69443,111 @@
       </c>
       <c r="M1598" s="4" t="s">
         <v>2416</v>
+      </c>
+    </row>
+    <row r="1599" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1599" s="4">
+        <v>620</v>
+      </c>
+      <c r="B1599" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1599" s="4">
+        <v>153310</v>
+      </c>
+      <c r="D1599" s="2" t="s">
+        <v>2598</v>
+      </c>
+      <c r="E1599" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1599" s="4" t="s">
+        <v>2599</v>
+      </c>
+      <c r="G1599" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1599" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1599" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1599" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1599" s="4" t="s">
+        <v>2502</v>
+      </c>
+    </row>
+    <row r="1600" spans="1:13" ht="150" x14ac:dyDescent="0.25">
+      <c r="A1600" s="4">
+        <v>621</v>
+      </c>
+      <c r="B1600" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1600" s="4">
+        <v>149511</v>
+      </c>
+      <c r="D1600" s="2" t="s">
+        <v>2598</v>
+      </c>
+      <c r="E1600" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1600" s="5" t="s">
+        <v>2600</v>
+      </c>
+      <c r="G1600" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1600" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I1600" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1600" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1600" s="4" t="s">
+        <v>2494</v>
+      </c>
+    </row>
+    <row r="1601" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1601" s="4">
+        <v>622</v>
+      </c>
+      <c r="B1601" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1601" s="4">
+        <v>140740</v>
+      </c>
+      <c r="D1601" s="2" t="s">
+        <v>2598</v>
+      </c>
+      <c r="E1601" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1601" s="4" t="s">
+        <v>2601</v>
+      </c>
+      <c r="G1601" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1601" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1601" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1601" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1601" s="4" t="s">
+        <v>2494</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 02/10/2026 19:40:47,29
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1580" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{867868CF-50ED-4178-A3BB-C643B59A8292}"/>
+  <xr:revisionPtr revIDLastSave="1597" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B180481A-C1CB-42A9-A656-43A982078139}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14496" uniqueCount="2602">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14532" uniqueCount="2608">
   <si>
     <t>ID</t>
   </si>
@@ -8097,6 +8097,28 @@
   </si>
   <si>
     <t>O serviço de agendamento e suporte ao cliente é muito problemático.</t>
+  </si>
+  <si>
+    <t>01/10/2026</t>
+  </si>
+  <si>
+    <t>02/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aqui só dei 5 pelo bom produto. Mas bom produto com serviço porco, vale pouco. Marquei a manutenção preventiva dia 21. Fiquei 5h esperando, visto que vocês não dão um horário e sim um periodo. Me deram o cano sem nenhuma explicação. Remarquei para dia 1/10 periodo tarde. Me programei para isso. Porem vieram pela manhã. Que tipo de atendimento é esse? Como vcs pioraram tanto? E o atendimento online é feito por pessoas totalmente despreparadas. </t>
+  </si>
+  <si>
+    <t>Marcaram à tarde, mas vieram pela manhã. Por acaso, era o dia da nossa diarista. Caso contrário não teria dado certo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Por incrível que pareça, agendei 4 (quatro) vezes no horário das 13:00 às 18:00 horas 
+Nenhuma vez cumpriram o horário agendado 
+Na quarta e última visita por uma coincidência terrível, o técnico de vcs chegou às 11:00 horas e eu estava em casa. A coordenação de vcs não estão em sintonia com os clientes.
+Meus parabéns equipe bem competente 
+Nota 3 pela marca Brastemp </t>
+  </si>
+  <si>
+    <t>Ficou faltando uma informação, avisei o atendente que de vez em quando na liberação de agua com gas não libera instantâneo, o painel fica acesso girando e tenho que esperar as vezes vários minutos para conseguir liberar agua com gas. Ele passou essa dúvida para central mais não teve retorno, será que não precisar trocar o aparelho?</t>
   </si>
 </sst>
 </file>
@@ -8552,7 +8574,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1601"/>
+  <dimension ref="A1:M1605"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -69550,6 +69572,146 @@
         <v>2494</v>
       </c>
     </row>
+    <row r="1602" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1602" s="4">
+        <v>623</v>
+      </c>
+      <c r="B1602" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1602" s="4">
+        <v>153268</v>
+      </c>
+      <c r="D1602" s="2" t="s">
+        <v>2602</v>
+      </c>
+      <c r="E1602" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1602" s="4" t="s">
+        <v>2604</v>
+      </c>
+      <c r="G1602" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1602" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1602" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1602" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1602" s="4" t="s">
+        <v>2492</v>
+      </c>
+    </row>
+    <row r="1603" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1603" s="4">
+        <v>624</v>
+      </c>
+      <c r="B1603" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1603" s="4">
+        <v>139312</v>
+      </c>
+      <c r="D1603" s="2" t="s">
+        <v>2602</v>
+      </c>
+      <c r="E1603" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1603" s="4" t="s">
+        <v>2605</v>
+      </c>
+      <c r="G1603" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1603" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1603" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1603" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1603" s="4" t="s">
+        <v>2416</v>
+      </c>
+    </row>
+    <row r="1604" spans="1:13" ht="135" x14ac:dyDescent="0.25">
+      <c r="A1604" s="4">
+        <v>625</v>
+      </c>
+      <c r="B1604" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1604" s="4">
+        <v>154874</v>
+      </c>
+      <c r="D1604" s="2" t="s">
+        <v>2603</v>
+      </c>
+      <c r="E1604" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1604" s="5" t="s">
+        <v>2606</v>
+      </c>
+      <c r="G1604" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1604" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1604" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1604" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1604" s="4" t="s">
+        <v>2492</v>
+      </c>
+    </row>
+    <row r="1605" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1605" s="4">
+        <v>626</v>
+      </c>
+      <c r="B1605" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1605" s="4">
+        <v>154819</v>
+      </c>
+      <c r="D1605" s="2" t="s">
+        <v>2603</v>
+      </c>
+      <c r="E1605" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1605" s="4" t="s">
+        <v>2607</v>
+      </c>
+      <c r="G1605" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1605" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1605" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1605" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1605" s="4" t="s">
+        <v>2452</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 05/10/2026 10:13:40,29
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1597" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B180481A-C1CB-42A9-A656-43A982078139}"/>
+  <xr:revisionPtr revIDLastSave="1627" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE007699-816D-475C-A825-FAD43DEE9A4E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14532" uniqueCount="2608">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14602" uniqueCount="2625">
   <si>
     <t>ID</t>
   </si>
@@ -8119,6 +8119,61 @@
   </si>
   <si>
     <t>Ficou faltando uma informação, avisei o atendente que de vez em quando na liberação de agua com gas não libera instantâneo, o painel fica acesso girando e tenho que esperar as vezes vários minutos para conseguir liberar agua com gas. Ele passou essa dúvida para central mais não teve retorno, será que não precisar trocar o aparelho?</t>
+  </si>
+  <si>
+    <t>03/10/2026</t>
+  </si>
+  <si>
+    <t>04/10/2026</t>
+  </si>
+  <si>
+    <t>05/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Porque na INSEGURANÇA em que vivemos,vocês DEIXARAM de continuar com o esquema de segurança que a Brastemp fazia,isto é enviava aos clientes antes do técnico chegar ,código da visita,nome e RG do funcionário que ia fazer o atendimento para ele .ser identificado por nós ,para poder ser feita sua identificação .Isso e’ feito pela Claro,Vivo e outras prestadoras de Serviço .
+Isso é muito simples de vocês implantarem .E’ só fazerem uma pequena inclusão no programa eletrônico de atendimento ao cliente .
+Quanto ao técnico ,seu trabalho foi excelente.
+Ah ,deixem conosco uma 2. Via do recibo do atendimento também.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Porque vcs priorizam o atendimento eletrônico em detrimento do pessoal, além de u ser há anos cliente e ter dois aparelhos em locais diferentes, pedi para um terceiro, mas, pedi um preço melhor , que me foi negado sem nenhuma atenção. </t>
+  </si>
+  <si>
+    <t>Só fui atendida como desejava depois de muito stress e visita que não aconteceu,  sem explicações. Quando desisti de me aborrecer, marcaram visita e por incrível que pareça,  fui atendida satisfatoriamente.</t>
+  </si>
+  <si>
+    <t>Marcou e não compareceu, depois marcou num horário e veio no outro.</t>
+  </si>
+  <si>
+    <t>Não vieram pela manhã como programado, a técnica não repos a etiqueta com as informações da última troca e contatos telefônico, deixou a copa toda respingada de água</t>
+  </si>
+  <si>
+    <t>Porque além de não resolver o problema inicial, ainda gerou estresse na hora de marcar nova data com o técnico.</t>
+  </si>
+  <si>
+    <t>FRQ LONDRINA PR R03</t>
+  </si>
+  <si>
+    <t>visita agendada não foi cumprida</t>
+  </si>
+  <si>
+    <t>não enviam dados do técnico + sem 2ª via do recibo</t>
+  </si>
+  <si>
+    <t>pedi preço melhor, negado + atendimento eletrônico</t>
+  </si>
+  <si>
+    <t>visita que não aconteceu, sem explicações</t>
+  </si>
+  <si>
+    <t>marcou e não compareceu + veio em outro horário</t>
+  </si>
+  <si>
+    <t>não vieram pela manhã + sem etiqueta + respingou água</t>
+  </si>
+  <si>
+    <t>não resolveu o problema inicial + estresse para remarcar</t>
   </si>
 </sst>
 </file>
@@ -8574,7 +8629,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1605"/>
+  <dimension ref="A1:M1611"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -67637,11 +67692,23 @@
       <c r="F1546" s="4" t="s">
         <v>1672</v>
       </c>
+      <c r="G1546" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1546" s="4" t="s">
+        <v>948</v>
+      </c>
       <c r="I1546" s="4" t="s">
         <v>1308</v>
       </c>
       <c r="J1546" s="4" t="s">
         <v>1337</v>
+      </c>
+      <c r="K1546" s="4" t="s">
+        <v>2618</v>
+      </c>
+      <c r="L1546" s="4" t="s">
+        <v>1550</v>
       </c>
       <c r="M1546" s="4" t="s">
         <v>2449</v>
@@ -69710,6 +69777,234 @@
       </c>
       <c r="M1605" s="4" t="s">
         <v>2452</v>
+      </c>
+    </row>
+    <row r="1606" spans="1:13" ht="225" x14ac:dyDescent="0.25">
+      <c r="B1606" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1606" s="4">
+        <v>138735</v>
+      </c>
+      <c r="D1606" s="2" t="s">
+        <v>2608</v>
+      </c>
+      <c r="E1606" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1606" s="5" t="s">
+        <v>2611</v>
+      </c>
+      <c r="G1606" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1606" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1606" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1606" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1606" s="4" t="s">
+        <v>2619</v>
+      </c>
+      <c r="L1606" s="4" t="s">
+        <v>1551</v>
+      </c>
+      <c r="M1606" s="4" t="s">
+        <v>2493</v>
+      </c>
+    </row>
+    <row r="1607" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B1607" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1607" s="4">
+        <v>150739</v>
+      </c>
+      <c r="D1607" s="2" t="s">
+        <v>2608</v>
+      </c>
+      <c r="E1607" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1607" s="4" t="s">
+        <v>2612</v>
+      </c>
+      <c r="G1607" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1607" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="I1607" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1607" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1607" s="4" t="s">
+        <v>2620</v>
+      </c>
+      <c r="L1607" s="4" t="s">
+        <v>1550</v>
+      </c>
+      <c r="M1607" s="4" t="s">
+        <v>2617</v>
+      </c>
+    </row>
+    <row r="1608" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B1608" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1608" s="4">
+        <v>148521</v>
+      </c>
+      <c r="D1608" s="2" t="s">
+        <v>2608</v>
+      </c>
+      <c r="E1608" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1608" s="4" t="s">
+        <v>2613</v>
+      </c>
+      <c r="G1608" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1608" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1608" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1608" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1608" s="4" t="s">
+        <v>2621</v>
+      </c>
+      <c r="L1608" s="4" t="s">
+        <v>1550</v>
+      </c>
+      <c r="M1608" s="4" t="s">
+        <v>2494</v>
+      </c>
+    </row>
+    <row r="1609" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B1609" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1609" s="4">
+        <v>155418</v>
+      </c>
+      <c r="D1609" s="2" t="s">
+        <v>2609</v>
+      </c>
+      <c r="E1609" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1609" s="4" t="s">
+        <v>2614</v>
+      </c>
+      <c r="G1609" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1609" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1609" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1609" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1609" s="4" t="s">
+        <v>2622</v>
+      </c>
+      <c r="L1609" s="4" t="s">
+        <v>1550</v>
+      </c>
+      <c r="M1609" s="4" t="s">
+        <v>2492</v>
+      </c>
+    </row>
+    <row r="1610" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B1610" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1610" s="4">
+        <v>152748</v>
+      </c>
+      <c r="D1610" s="2" t="s">
+        <v>2610</v>
+      </c>
+      <c r="E1610" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1610" s="4" t="s">
+        <v>2615</v>
+      </c>
+      <c r="G1610" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1610" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1610" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1610" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1610" s="4" t="s">
+        <v>2623</v>
+      </c>
+      <c r="L1610" s="4" t="s">
+        <v>1551</v>
+      </c>
+      <c r="M1610" s="4" t="s">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="1611" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B1611" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1611" s="4">
+        <v>156293</v>
+      </c>
+      <c r="D1611" s="2" t="s">
+        <v>2610</v>
+      </c>
+      <c r="E1611" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1611" s="4" t="s">
+        <v>2616</v>
+      </c>
+      <c r="G1611" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1611" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1611" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1611" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1611" s="4" t="s">
+        <v>2624</v>
+      </c>
+      <c r="L1611" s="4" t="s">
+        <v>1550</v>
+      </c>
+      <c r="M1611" s="4" t="s">
+        <v>2492</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 08/10/2026 11:10:37,15
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2716" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{26A3224E-F964-4036-90E8-448D27AEF531}"/>
+  <xr:revisionPtr revIDLastSave="2823" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0845E1C-C723-4542-BC4D-36F593934B1A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$1570</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$M$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16290" uniqueCount="3387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16326" uniqueCount="3396">
   <si>
     <t>ID</t>
   </si>
@@ -10466,6 +10466,34 @@
   </si>
   <si>
     <t>não ajustou fluxo, estava vazando + sem ferramenta</t>
+  </si>
+  <si>
+    <t>07/10/2026</t>
+  </si>
+  <si>
+    <t>08/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">demora para limpeza do filtro </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marquei a visita do  técnico para a manutenção técnica do purificador e ele não veio
+</t>
+  </si>
+  <si>
+    <t>Desde que a Culligan assumiu só tive problemas. Ficaram 3 meses sem cobrar, não avisaram do atraso, depois mudaram o dia do pagamento e fiquei novamente em atraso pois não fui informada e na data X ñao tinha dinheiro na conta, Mandaram Whatsapp para marcar a manutenção, chegou no dia não veio ninguém. Tudo isso qdo reclamo falam que eh erro do sistema. E outra, antes podíamos marcar a manutenção e/ou problema com uma no max estourando 2 semanas. Agora para marcar a manutenção é um mês pra frente. O que está havendo? Sou cliente a mais de 10 anos da Brastemp e na gestão Whillor (ANTERIOR A CULLIGAN) isso não acontecia! Péssima troca. Péssima troca!!!! Precisam rever isso. E vou averiguar agora, se nnao vou.ve cobrança em duplicidade, pq nunca vi uma empresa mudar data de pagamento em debito automático sem avisar, sem notificar. Péssimo , péssimo!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Porque desde que o purificador brastemp que  tenho a mais de 10 anos passou para a Culligan , nada funciona , as marcações de visita não são respeitadas , a cobrança saiu do débito automático e não mandam o boleto para pagamento. Já solicitei várias vezes e só consigo falar com robô . </t>
+  </si>
+  <si>
+    <t>FRQ SANTOS SP R02</t>
+  </si>
+  <si>
+    <t>Financeiro</t>
+  </si>
+  <si>
+    <t>Problemas no Faturamento</t>
   </si>
 </sst>
 </file>
@@ -10921,7 +10949,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1625"/>
+  <dimension ref="A1:M1629"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -17315,10 +17343,10 @@
         <v>190</v>
       </c>
       <c r="G156" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H156" s="4" t="s">
-        <v>66</v>
+        <v>3395</v>
       </c>
       <c r="I156" s="4" t="s">
         <v>1307</v>
@@ -22153,10 +22181,10 @@
         <v>310</v>
       </c>
       <c r="G274" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H274" s="4" t="s">
-        <v>66</v>
+        <v>3395</v>
       </c>
       <c r="I274" s="4" t="s">
         <v>1307</v>
@@ -22276,10 +22304,10 @@
         <v>313</v>
       </c>
       <c r="G277" s="4" t="s">
-        <v>25</v>
+        <v>3394</v>
       </c>
       <c r="H277" s="4" t="s">
-        <v>26</v>
+        <v>3395</v>
       </c>
       <c r="I277" s="4" t="s">
         <v>1307</v>
@@ -34822,10 +34850,10 @@
         <v>619</v>
       </c>
       <c r="G583" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H583" s="4" t="s">
-        <v>133</v>
+        <v>3395</v>
       </c>
       <c r="I583" s="4" t="s">
         <v>1307</v>
@@ -35724,10 +35752,10 @@
         <v>641</v>
       </c>
       <c r="G605" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H605" s="4" t="s">
-        <v>392</v>
+        <v>3395</v>
       </c>
       <c r="I605" s="4" t="s">
         <v>1307</v>
@@ -37077,10 +37105,10 @@
         <v>673</v>
       </c>
       <c r="G638" s="4" t="s">
-        <v>25</v>
+        <v>3394</v>
       </c>
       <c r="H638" s="4" t="s">
-        <v>26</v>
+        <v>3395</v>
       </c>
       <c r="I638" s="4" t="s">
         <v>1307</v>
@@ -43473,10 +43501,10 @@
         <v>829</v>
       </c>
       <c r="G794" s="4" t="s">
-        <v>134</v>
+        <v>3394</v>
       </c>
       <c r="H794" s="4" t="s">
-        <v>158</v>
+        <v>3395</v>
       </c>
       <c r="I794" s="4" t="s">
         <v>1307</v>
@@ -44949,10 +44977,10 @@
         <v>864</v>
       </c>
       <c r="G830" s="4" t="s">
-        <v>15</v>
+        <v>3394</v>
       </c>
       <c r="H830" s="4" t="s">
-        <v>40</v>
+        <v>3395</v>
       </c>
       <c r="I830" s="4" t="s">
         <v>1307</v>
@@ -45851,10 +45879,10 @@
         <v>886</v>
       </c>
       <c r="G852" s="4" t="s">
-        <v>28</v>
+        <v>3394</v>
       </c>
       <c r="H852" s="4" t="s">
-        <v>200</v>
+        <v>3395</v>
       </c>
       <c r="I852" s="4" t="s">
         <v>1307</v>
@@ -46056,10 +46084,10 @@
         <v>891</v>
       </c>
       <c r="G857" s="4" t="s">
-        <v>15</v>
+        <v>3394</v>
       </c>
       <c r="H857" s="4" t="s">
-        <v>18</v>
+        <v>3395</v>
       </c>
       <c r="I857" s="4" t="s">
         <v>1307</v>
@@ -48106,10 +48134,10 @@
         <v>941</v>
       </c>
       <c r="G907" s="4" t="s">
-        <v>51</v>
+        <v>3394</v>
       </c>
       <c r="H907" s="4" t="s">
-        <v>2769</v>
+        <v>3395</v>
       </c>
       <c r="I907" s="4" t="s">
         <v>1307</v>
@@ -53928,10 +53956,10 @@
         <v>1082</v>
       </c>
       <c r="G1049" s="4" t="s">
-        <v>15</v>
+        <v>3394</v>
       </c>
       <c r="H1049" s="4" t="s">
-        <v>40</v>
+        <v>3395</v>
       </c>
       <c r="I1049" s="4" t="s">
         <v>1307</v>
@@ -54051,10 +54079,10 @@
         <v>1085</v>
       </c>
       <c r="G1052" s="4" t="s">
-        <v>15</v>
+        <v>3394</v>
       </c>
       <c r="H1052" s="4" t="s">
-        <v>948</v>
+        <v>3395</v>
       </c>
       <c r="I1052" s="4" t="s">
         <v>1307</v>
@@ -56224,10 +56252,10 @@
         <v>1137</v>
       </c>
       <c r="G1105" s="4" t="s">
-        <v>11</v>
+        <v>3394</v>
       </c>
       <c r="H1105" s="4" t="s">
-        <v>21</v>
+        <v>3395</v>
       </c>
       <c r="I1105" s="4" t="s">
         <v>1307</v>
@@ -56429,10 +56457,10 @@
         <v>1142</v>
       </c>
       <c r="G1110" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H1110" s="4" t="s">
-        <v>66</v>
+        <v>3395</v>
       </c>
       <c r="I1110" s="4" t="s">
         <v>1307</v>
@@ -58971,10 +58999,10 @@
         <v>1203</v>
       </c>
       <c r="G1172" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H1172" s="4" t="s">
-        <v>133</v>
+        <v>3395</v>
       </c>
       <c r="I1172" s="4" t="s">
         <v>1307</v>
@@ -62333,10 +62361,10 @@
         <v>1284</v>
       </c>
       <c r="G1254" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H1254" s="4" t="s">
-        <v>133</v>
+        <v>3395</v>
       </c>
       <c r="I1254" s="4" t="s">
         <v>1308</v>
@@ -63358,10 +63386,10 @@
         <v>1312</v>
       </c>
       <c r="G1279" s="4" t="s">
-        <v>15</v>
+        <v>3394</v>
       </c>
       <c r="H1279" s="4" t="s">
-        <v>18</v>
+        <v>3395</v>
       </c>
       <c r="I1279" s="4" t="s">
         <v>1307</v>
@@ -63891,10 +63919,10 @@
         <v>1326</v>
       </c>
       <c r="G1292" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H1292" s="4" t="s">
-        <v>133</v>
+        <v>3395</v>
       </c>
       <c r="I1292" s="4" t="s">
         <v>1308</v>
@@ -65162,10 +65190,10 @@
         <v>1365</v>
       </c>
       <c r="G1323" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H1323" s="4" t="s">
-        <v>133</v>
+        <v>3395</v>
       </c>
       <c r="I1323" s="4" t="s">
         <v>1308</v>
@@ -65613,10 +65641,10 @@
         <v>1376</v>
       </c>
       <c r="G1334" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H1334" s="4" t="s">
-        <v>133</v>
+        <v>3395</v>
       </c>
       <c r="I1334" s="4" t="s">
         <v>1308</v>
@@ -66351,10 +66379,10 @@
         <v>1394</v>
       </c>
       <c r="G1352" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H1352" s="4" t="s">
-        <v>133</v>
+        <v>3395</v>
       </c>
       <c r="I1352" s="4" t="s">
         <v>1308</v>
@@ -67007,10 +67035,10 @@
         <v>1410</v>
       </c>
       <c r="G1368" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H1368" s="4" t="s">
-        <v>66</v>
+        <v>3395</v>
       </c>
       <c r="I1368" s="4" t="s">
         <v>1308</v>
@@ -67540,10 +67568,10 @@
         <v>1417</v>
       </c>
       <c r="G1381" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H1381" s="4" t="s">
-        <v>133</v>
+        <v>3395</v>
       </c>
       <c r="I1381" s="4" t="s">
         <v>1422</v>
@@ -68114,10 +68142,10 @@
         <v>1439</v>
       </c>
       <c r="G1395" s="4" t="s">
-        <v>15</v>
+        <v>3394</v>
       </c>
       <c r="H1395" s="4" t="s">
-        <v>18</v>
+        <v>3395</v>
       </c>
       <c r="I1395" s="4" t="s">
         <v>1308</v>
@@ -68278,10 +68306,10 @@
         <v>1443</v>
       </c>
       <c r="G1399" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H1399" s="4" t="s">
-        <v>66</v>
+        <v>3395</v>
       </c>
       <c r="I1399" s="4" t="s">
         <v>1308</v>
@@ -68606,10 +68634,10 @@
         <v>1451</v>
       </c>
       <c r="G1407" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H1407" s="4" t="s">
-        <v>133</v>
+        <v>3395</v>
       </c>
       <c r="I1407" s="4" t="s">
         <v>1308</v>
@@ -68688,10 +68716,10 @@
         <v>1453</v>
       </c>
       <c r="G1409" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H1409" s="4" t="s">
-        <v>392</v>
+        <v>3395</v>
       </c>
       <c r="I1409" s="4" t="s">
         <v>1308</v>
@@ -69180,10 +69208,10 @@
         <v>1467</v>
       </c>
       <c r="G1421" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H1421" s="4" t="s">
-        <v>66</v>
+        <v>3395</v>
       </c>
       <c r="I1421" s="4" t="s">
         <v>1308</v>
@@ -69344,10 +69372,10 @@
         <v>1460</v>
       </c>
       <c r="G1425" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H1425" s="4" t="s">
-        <v>66</v>
+        <v>3395</v>
       </c>
       <c r="I1425" s="4" t="s">
         <v>1308</v>
@@ -70861,10 +70889,10 @@
         <v>1508</v>
       </c>
       <c r="G1462" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H1462" s="4" t="s">
-        <v>66</v>
+        <v>3395</v>
       </c>
       <c r="I1462" s="4" t="s">
         <v>1308</v>
@@ -71107,10 +71135,10 @@
         <v>1515</v>
       </c>
       <c r="G1468" s="4" t="s">
-        <v>15</v>
+        <v>3394</v>
       </c>
       <c r="H1468" s="4" t="s">
-        <v>948</v>
+        <v>3395</v>
       </c>
       <c r="I1468" s="4" t="s">
         <v>1308</v>
@@ -73157,10 +73185,10 @@
         <v>1611</v>
       </c>
       <c r="G1518" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H1518" s="4" t="s">
-        <v>66</v>
+        <v>3395</v>
       </c>
       <c r="I1518" s="4" t="s">
         <v>1308</v>
@@ -74756,10 +74784,10 @@
         <v>2536</v>
       </c>
       <c r="G1557" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H1557" s="4" t="s">
-        <v>133</v>
+        <v>3395</v>
       </c>
       <c r="I1557" s="4" t="s">
         <v>1308</v>
@@ -75289,10 +75317,10 @@
         <v>2554</v>
       </c>
       <c r="G1570" s="4" t="s">
-        <v>28</v>
+        <v>3394</v>
       </c>
       <c r="H1570" s="4" t="s">
-        <v>81</v>
+        <v>3395</v>
       </c>
       <c r="I1570" s="4" t="s">
         <v>1308</v>
@@ -75740,10 +75768,10 @@
         <v>2569</v>
       </c>
       <c r="G1581" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H1581" s="4" t="s">
-        <v>66</v>
+        <v>3395</v>
       </c>
       <c r="I1581" s="4" t="s">
         <v>1308</v>
@@ -76232,10 +76260,10 @@
         <v>2585</v>
       </c>
       <c r="G1593" s="4" t="s">
-        <v>65</v>
+        <v>3394</v>
       </c>
       <c r="H1593" s="4" t="s">
-        <v>133</v>
+        <v>3395</v>
       </c>
       <c r="I1593" s="4" t="s">
         <v>1308</v>
@@ -76314,10 +76342,10 @@
         <v>2587</v>
       </c>
       <c r="G1595" s="4" t="s">
-        <v>25</v>
+        <v>3394</v>
       </c>
       <c r="H1595" s="4" t="s">
-        <v>26</v>
+        <v>3395</v>
       </c>
       <c r="I1595" s="4" t="s">
         <v>1308</v>
@@ -77298,10 +77326,10 @@
         <v>2611</v>
       </c>
       <c r="G1619" s="4" t="s">
-        <v>15</v>
+        <v>3394</v>
       </c>
       <c r="H1619" s="4" t="s">
-        <v>948</v>
+        <v>3395</v>
       </c>
       <c r="I1619" s="4" t="s">
         <v>1308</v>
@@ -77565,7 +77593,136 @@
         <v>2494</v>
       </c>
     </row>
+    <row r="1626" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B1626" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1626" s="4">
+        <v>158917</v>
+      </c>
+      <c r="D1626" s="2" t="s">
+        <v>3387</v>
+      </c>
+      <c r="E1626" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1626" s="4" t="s">
+        <v>3389</v>
+      </c>
+      <c r="G1626" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1626" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1626" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1626" s="4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="M1626" s="4" t="s">
+        <v>2487</v>
+      </c>
+    </row>
+    <row r="1627" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B1627" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1627" s="4">
+        <v>159122</v>
+      </c>
+      <c r="D1627" s="2" t="s">
+        <v>3387</v>
+      </c>
+      <c r="E1627" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1627" s="4" t="s">
+        <v>3390</v>
+      </c>
+      <c r="G1627" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1627" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1627" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1627" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1627" s="4" t="s">
+        <v>2495</v>
+      </c>
+    </row>
+    <row r="1628" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B1628" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1628" s="4">
+        <v>161524</v>
+      </c>
+      <c r="D1628" s="2" t="s">
+        <v>3387</v>
+      </c>
+      <c r="E1628" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1628" s="4" t="s">
+        <v>3391</v>
+      </c>
+      <c r="G1628" s="4" t="s">
+        <v>3394</v>
+      </c>
+      <c r="H1628" s="4" t="s">
+        <v>3395</v>
+      </c>
+      <c r="I1628" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1628" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1628" s="4" t="s">
+        <v>3393</v>
+      </c>
+    </row>
+    <row r="1629" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B1629" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1629" s="4">
+        <v>160872</v>
+      </c>
+      <c r="D1629" s="2" t="s">
+        <v>3388</v>
+      </c>
+      <c r="E1629" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1629" s="4" t="s">
+        <v>3392</v>
+      </c>
+      <c r="G1629" s="4" t="s">
+        <v>3394</v>
+      </c>
+      <c r="H1629" s="4" t="s">
+        <v>3395</v>
+      </c>
+      <c r="I1629" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1629" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1629" s="4" t="s">
+        <v>2410</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:M1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 14/10/2026  9:01:17,75
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2848" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4AD39BB3-6A9B-4E0A-8035-F5C485078235}"/>
+  <xr:revisionPtr revIDLastSave="2867" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5ADB7116-F99D-4A6D-B1FA-5DE68608FF84}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16366" uniqueCount="3402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16624" uniqueCount="3459">
   <si>
     <t>ID</t>
   </si>
@@ -10519,6 +10519,190 @@
   </si>
   <si>
     <t>campo</t>
+  </si>
+  <si>
+    <t>FRQ BRASILIA DF R04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O filtro instalado já foi instalado com defeito e a troca do filtro só será feita dia 20 tenho 2 idosos em casa </t>
+  </si>
+  <si>
+    <t>Pela segunda vez seguida, a visita e manutenção foi marcada para o horário da tarde e o técnico apareceu pela manhã. Na primeira vez, no ano passado, foi necessário remarcar. Neste ano, por acaso tinha alguém em casa, que pôde acompanhar a visita.</t>
+  </si>
+  <si>
+    <t>Hoje o técnico compareceu em nossa unidade para realizar a preventiva apenas de "1 purificador" os outros 2 ficaram sem reparo, a etiqueta consta vencido em setembro; Ficamos no aguardo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desde que passou para a Culligan e tiraram o pagamento do débito automático, tenho tido problemas para pagar a mensalidade. É trabalhoso, desgastante, muito tempo esperando ao telefone, tocando m[usica, antes de transferir para o financeiro, 10:07, atendem e nao conseguem me enviar  boleto do pagamento.´e muito estressante. Quando atendem, desligam o telefone!!
+Hoje,neste momento. é a terceira vez que ligo, Evely, Samuel e outra atendente, última agoa. esqueci o nome, mal conseguia falar, caia a ligação ou eles desligaram o telefone!
+É uma falta de respeito e consideração um atendimento ao cliente,como esse. Obrigada. </t>
+  </si>
+  <si>
+    <t>Pq meu problema não foi resolvido, e o técnico solicitou a troca do aparelho, que foi agendado para o dia 24/10. 
+Até lá vamos ficar sem usar o purificador.
+Porque não está saindo agua gelada,  nem fria, e a natural esta quente.</t>
+  </si>
+  <si>
+    <t>A data disponível para agendamento de visita técnica destinada a conserto de um defeito foi muito distante. Pedi prioridade mas não atenderam, embora seja um bom e antigo cliente. Fiquei uma semana sem utilizar o purificador e tive gasto com a compra de água mineral.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A água não está saindo gelado EA natural está saindo quente </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Devido ao atendimento da area juridica - contratos.
+Quando da mudança de Brastemp para Culligan nos orientaram a fazer um adendo ao contrato.
+Gerou-se esforços desnecessários, pois aoi final do processo uma das pessoas da Culligan não assinou o documento e informaram que não era mais necessário.
+Essa situação foi muito desagradável.
+Quanto ao produto locado não tenho qualquer comentário.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não cumpriram o horário da visita para manutenção, além do que não trouxeram o equipamento para resolver a baixa pressão. </t>
+  </si>
+  <si>
+    <t>Foi uma técnica fazer a visita periódica no dia 25/09, disse que só fez o teste da água, mas desde que ela saiu, o filtro na sai água na opção gelada e bem na com gás. Só foi possível marcar outra visita para o dia 02/10. O técnico disse que tinha queimado alguma coisa e disse que trocou. Porém continua com os mesmos problemas. Liguei para pedir uma visita com urgência e só consegui agendar para o dia 08/10. Ou seja, vai totalizar 2 semanas sem água gelada (motivo pelo qual fechei com vocês) e nessa visita vai acabar sendo a mesma coisa, vai vir uma pessoa, trocar uma coisinha e cair fora. Eles não esperam a água gelada sair para ir embora e ver que realmente deu certo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eu avaliei o atendimento com um especialista com o máximo,  porém expliquei que reformei a cozinha e que tinha que reinstalar o purificador. Chegou o técnico apenas para manutenção. Provei pela conversa no WhatsApp que não era só manutenção.  Tempo perdido. A OS era só manutenção! Sem obs alguma inclusive que a mangueira deveria ter 1,5m. NÃO FOI FEITA A MANUTENÇÃO </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Além de todos os problemas até a data da manutenção, no dia marcado o horário não foi cumprido. Atenção parece que o funcionário não foi culpado pois segundo ele havia grande número de visitas </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chegou antes do horário agendado </t>
+  </si>
+  <si>
+    <t>Foi muito estranho!!!! Agendei pelo WhatsApp p dia 13 out pela manhã e vieram sem avisar no dia 8 out!!!!</t>
+  </si>
+  <si>
+    <t>As manutenções regulares não foram realizadas nas datas agendas por 3 vezes seguidas. A visita foi realizada apenas após eu tentar cancelar o serviço.  O técnico veio realizar a visita em um dia diferente do combinado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intalou mas deu vazamento em baixo </t>
+  </si>
+  <si>
+    <t>Atendimento muito impessoal, não ouve o cliente, fiz um agendamento de rotina, chegou aqui um  técnico que tinha um chamado de manutenção, não fez nada, abriu e fechou a torneira e foi embora, não tenho certeza se esse filtro precisa ou não de reparo, o técnico se quer pode explicar tamanha a pressa que ele tinha de sair.</t>
+  </si>
+  <si>
+    <t>O serviço não foi realizado. Agendei entre 13 e 18hs, o técnico apareceu as 12hs, fora do horário marcado. Marquei após as 13hs justamente porque não podia atender antes. Solicitei ao porteiro que informasse ao técnico a impossibilidade, e que o mesmo retornasse ao intervalo anteriormente marcado, o que não aconteceu.  Péssimo serviço!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demoram demais para fazer visita e quando fazem sempre falam que não precisa trocar o filtro. Engraçado.. se eu tivesse que comprar.. teria que trocar de 3 em 3 meses. Como pago mensalidade, querem trocar 1 vez por ano e olhe lá. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">pq pela 4a, 5a vez já havia solicitado a "troca do aparelho", conf minha assinatura + de 08 anos e sempre a mesma desculpa, o técnico chega diz que n tem nenhuma observação p troca, q a mesma deve ser solicitada etc...a história se repete, o tempo passa, meu aparelho talvez nem tenha + atualização, peças de substituição s demoradas. Essa mensagem n diz respeito aos atendimentos pessoais, os técnicos enviados n tem culpa, eles simplesmente atendem o que é passado e exatamente o que passam como simples manutenção que deve ser reavaliado. No mesmo dia, 3 reclamações no mesmo condominio, pelo mesmo motivo . </t>
+  </si>
+  <si>
+    <t>Eu gosto do filtro e da qualidade ! A minha nota diz respeito a visita que é agendada, porém o técnico não cumpre o horário, já é a segunda vez que isso ocorre! Na visita anterior ele não veio tive que reagendar. Hj, qdo reclamei, recebi uma ligação e logo em seguida o interfone tocou dizendo que ele havia chegado, muito estranho isso, ele trocou o filtro em menos de 5 minutos! A gente desmarca compromissos e fica esperando. Melhor vcs agendarem um horário e não um período, facilitaria muito.</t>
+  </si>
+  <si>
+    <t>Péssima qualidade na comunicação entre funcionários e clientes. Qto ao purificador é ótimo mas o funcionamento da empresa NÃO É BOM! São enrolados. O funcionário veio aqui trocar o filtro e a água não está como das outras vezes.... tá com gosto ruim. Vou esperar mais uns 2 dias p ver se melhora o gosto.</t>
+  </si>
+  <si>
+    <t>Olá!
+O atendimento foi bom, porém fiquei bastante insatisfeito com a substituição do equipamento. O aparelho disponibilizado, além de ser recondicionado, é de um modelo inferior ao que eu tinha anteriormente, o que considero uma perda na qualidade do serviço contratado.
+Dessa forma, peço que avaliem a situação e considerem a possibilidade de retornar com o modelo do equipamento anterior, pois, nas condições atuais, não estou satisfeito com o serviço da Brastemp Culligan.
+Caso não seja possível solucionar essa questão, infelizmente terei que cancelar minha assinatura.
+Aguardo um retorno e uma solução para o caso. Obrigado.</t>
+  </si>
+  <si>
+    <t>demora para limpeza do filtro</t>
+  </si>
+  <si>
+    <t>marquei a visita e ele não veio</t>
+  </si>
+  <si>
+    <t>mudaram data do débito + visita não veio + agenda distante</t>
+  </si>
+  <si>
+    <t>saiu do débito automático, sem boleto + visitas não respeitadas</t>
+  </si>
+  <si>
+    <t>filtro não é mais trocado semestralmente</t>
+  </si>
+  <si>
+    <t>serviço não ficou perfeito (genérico)</t>
+  </si>
+  <si>
+    <t>ninguém apareceu no segundo endereço</t>
+  </si>
+  <si>
+    <t>troca só dia 20 + instalado com defeito</t>
+  </si>
+  <si>
+    <t>marcado à tarde, apareceu pela manhã</t>
+  </si>
+  <si>
+    <t>preventiva de apenas 1 de 3 purificadores</t>
+  </si>
+  <si>
+    <t>tiraram débito automático + atendimento telefônico ruim</t>
+  </si>
+  <si>
+    <t>troca agendada só 24/10 + não gela</t>
+  </si>
+  <si>
+    <t>data para visita técnica muito distante</t>
+  </si>
+  <si>
+    <t>"Bom" (comentário positivo, nota detratora)</t>
+  </si>
+  <si>
+    <t>água não sai gelada, natural quente</t>
+  </si>
+  <si>
+    <t>orientaram adendo, depois não era necessário</t>
+  </si>
+  <si>
+    <t>não trouxeram equipamento + horário não cumprido</t>
+  </si>
+  <si>
+    <t>continua com os mesmos problemas + agenda 08/10 + só testou</t>
+  </si>
+  <si>
+    <t>OS só manutenção, pedido era reinstalação</t>
+  </si>
+  <si>
+    <t>no dia marcado o horário não foi cumprido</t>
+  </si>
+  <si>
+    <t>chegou antes do horário agendado</t>
+  </si>
+  <si>
+    <t>agendado dia 13, vieram sem avisar dia 8</t>
+  </si>
+  <si>
+    <t>não realizadas nas datas 3 vezes + dia diferente</t>
+  </si>
+  <si>
+    <t>instalou mas deu vazamento embaixo</t>
+  </si>
+  <si>
+    <t>abriu e fechou a torneira e foi embora</t>
+  </si>
+  <si>
+    <t>técnico apareceu às 12h, fora do horário</t>
+  </si>
+  <si>
+    <t>não trocam o filtro + demora na visita</t>
+  </si>
+  <si>
+    <t>pela 4ª, 5ª vez solicitei a troca</t>
+  </si>
+  <si>
+    <t>técnico não cumpre horário + não veio antes + 5 min</t>
+  </si>
+  <si>
+    <t>gosto ruim após troca do filtro + comunicação ruim</t>
+  </si>
+  <si>
+    <t>recondicionado e modelo inferior ao anterior</t>
+  </si>
+  <si>
+    <t>parou de gelar após a visita + ruído</t>
+  </si>
+  <si>
+    <t>mangueira insuficiente + promessa na venda</t>
   </si>
 </sst>
 </file>
@@ -10974,7 +11158,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1634"/>
+  <dimension ref="A1:M1658"/>
   <sheetFormatPr defaultRowHeight="24" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -77649,6 +77833,12 @@
       <c r="J1626" s="4" t="s">
         <v>1338</v>
       </c>
+      <c r="K1626" s="4" t="s">
+        <v>3426</v>
+      </c>
+      <c r="L1626" s="4" t="s">
+        <v>1547</v>
+      </c>
       <c r="M1626" s="4" t="s">
         <v>2487</v>
       </c>
@@ -77684,6 +77874,12 @@
       <c r="J1627" s="4" t="s">
         <v>1337</v>
       </c>
+      <c r="K1627" s="4" t="s">
+        <v>3427</v>
+      </c>
+      <c r="L1627" s="4" t="s">
+        <v>1546</v>
+      </c>
       <c r="M1627" s="4" t="s">
         <v>2495</v>
       </c>
@@ -77719,6 +77915,12 @@
       <c r="J1628" s="4" t="s">
         <v>1337</v>
       </c>
+      <c r="K1628" s="4" t="s">
+        <v>3428</v>
+      </c>
+      <c r="L1628" s="4" t="s">
+        <v>1547</v>
+      </c>
       <c r="M1628" s="4" t="s">
         <v>3393</v>
       </c>
@@ -77754,6 +77956,12 @@
       <c r="J1629" s="4" t="s">
         <v>1337</v>
       </c>
+      <c r="K1629" s="4" t="s">
+        <v>3429</v>
+      </c>
+      <c r="L1629" s="4" t="s">
+        <v>1547</v>
+      </c>
       <c r="M1629" s="4" t="s">
         <v>2410</v>
       </c>
@@ -77789,6 +77997,12 @@
       <c r="J1630" s="4" t="s">
         <v>1337</v>
       </c>
+      <c r="K1630" s="4" t="s">
+        <v>3430</v>
+      </c>
+      <c r="L1630" s="4" t="s">
+        <v>1546</v>
+      </c>
       <c r="M1630" s="4" t="s">
         <v>2485</v>
       </c>
@@ -77824,6 +78038,12 @@
       <c r="J1631" s="4" t="s">
         <v>1337</v>
       </c>
+      <c r="K1631" s="4" t="s">
+        <v>3431</v>
+      </c>
+      <c r="L1631" s="4" t="s">
+        <v>1547</v>
+      </c>
       <c r="M1631" s="4" t="s">
         <v>2492</v>
       </c>
@@ -77859,6 +78079,12 @@
       <c r="J1632" s="4" t="s">
         <v>1337</v>
       </c>
+      <c r="K1632" s="4" t="s">
+        <v>3432</v>
+      </c>
+      <c r="L1632" s="4" t="s">
+        <v>1546</v>
+      </c>
       <c r="M1632" s="4" t="s">
         <v>2494</v>
       </c>
@@ -77894,6 +78120,12 @@
       <c r="J1633" s="4" t="s">
         <v>1337</v>
       </c>
+      <c r="K1633" s="4" t="s">
+        <v>3457</v>
+      </c>
+      <c r="L1633" s="4" t="s">
+        <v>1547</v>
+      </c>
       <c r="M1633" s="4" t="s">
         <v>2512</v>
       </c>
@@ -77929,12 +78161,1001 @@
       <c r="J1634" s="4" t="s">
         <v>1337</v>
       </c>
+      <c r="K1634" s="4" t="s">
+        <v>3458</v>
+      </c>
+      <c r="L1634" s="4" t="s">
+        <v>1547</v>
+      </c>
       <c r="M1634" s="4" t="s">
         <v>2495</v>
       </c>
     </row>
+    <row r="1635" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1635" s="4">
+        <v>656</v>
+      </c>
+      <c r="B1635" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1635" s="4">
+        <v>162940</v>
+      </c>
+      <c r="D1635" s="2">
+        <v>46304</v>
+      </c>
+      <c r="E1635" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1635" s="4" t="s">
+        <v>3403</v>
+      </c>
+      <c r="G1635" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1635" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1635" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1635" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1635" s="4" t="s">
+        <v>3433</v>
+      </c>
+      <c r="L1635" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1635" s="4" t="s">
+        <v>2488</v>
+      </c>
+    </row>
+    <row r="1636" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1636" s="4">
+        <v>657</v>
+      </c>
+      <c r="B1636" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1636" s="4">
+        <v>160726</v>
+      </c>
+      <c r="D1636" s="2">
+        <v>46304</v>
+      </c>
+      <c r="E1636" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1636" s="4" t="s">
+        <v>3404</v>
+      </c>
+      <c r="G1636" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1636" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1636" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1636" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1636" s="4" t="s">
+        <v>3434</v>
+      </c>
+      <c r="L1636" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1636" s="4" t="s">
+        <v>2410</v>
+      </c>
+    </row>
+    <row r="1637" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1637" s="4">
+        <v>658</v>
+      </c>
+      <c r="B1637" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1637" s="4">
+        <v>162386</v>
+      </c>
+      <c r="D1637" s="2">
+        <v>46304</v>
+      </c>
+      <c r="E1637" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1637" s="4" t="s">
+        <v>3405</v>
+      </c>
+      <c r="G1637" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1637" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I1637" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1637" s="4" t="s">
+        <v>1359</v>
+      </c>
+      <c r="K1637" s="4" t="s">
+        <v>3435</v>
+      </c>
+      <c r="L1637" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1637" s="4" t="s">
+        <v>2485</v>
+      </c>
+    </row>
+    <row r="1638" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1638" s="4">
+        <v>659</v>
+      </c>
+      <c r="B1638" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1638" s="4">
+        <v>150173</v>
+      </c>
+      <c r="D1638" s="2">
+        <v>46304</v>
+      </c>
+      <c r="E1638" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1638" s="4" t="s">
+        <v>3406</v>
+      </c>
+      <c r="G1638" s="4" t="s">
+        <v>3394</v>
+      </c>
+      <c r="H1638" s="4" t="s">
+        <v>3395</v>
+      </c>
+      <c r="I1638" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1638" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1638" s="4" t="s">
+        <v>3436</v>
+      </c>
+      <c r="L1638" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1638" s="4" t="s">
+        <v>2506</v>
+      </c>
+    </row>
+    <row r="1639" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1639" s="4">
+        <v>660</v>
+      </c>
+      <c r="B1639" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1639" s="4">
+        <v>160209</v>
+      </c>
+      <c r="D1639" s="2">
+        <v>46304</v>
+      </c>
+      <c r="E1639" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1639" s="4" t="s">
+        <v>3407</v>
+      </c>
+      <c r="G1639" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1639" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1639" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1639" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1639" s="4" t="s">
+        <v>3437</v>
+      </c>
+      <c r="L1639" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1639" s="4" t="s">
+        <v>2443</v>
+      </c>
+    </row>
+    <row r="1640" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1640" s="4">
+        <v>661</v>
+      </c>
+      <c r="B1640" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1640" s="4">
+        <v>158919</v>
+      </c>
+      <c r="D1640" s="2">
+        <v>46304</v>
+      </c>
+      <c r="E1640" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1640" s="4" t="s">
+        <v>3408</v>
+      </c>
+      <c r="G1640" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1640" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1640" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1640" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1640" s="4" t="s">
+        <v>3438</v>
+      </c>
+      <c r="L1640" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1640" s="4" t="s">
+        <v>3402</v>
+      </c>
+    </row>
+    <row r="1641" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1641" s="4">
+        <v>662</v>
+      </c>
+      <c r="B1641" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1641" s="4">
+        <v>159170</v>
+      </c>
+      <c r="D1641" s="2">
+        <v>46304</v>
+      </c>
+      <c r="E1641" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1641" s="4" t="s">
+        <v>448</v>
+      </c>
+      <c r="G1641" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1641" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1641" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1641" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1641" s="4" t="s">
+        <v>3439</v>
+      </c>
+      <c r="L1641" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1641" s="4" t="s">
+        <v>2492</v>
+      </c>
+    </row>
+    <row r="1642" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1642" s="4">
+        <v>663</v>
+      </c>
+      <c r="B1642" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1642" s="4">
+        <v>161157</v>
+      </c>
+      <c r="D1642" s="2">
+        <v>46304</v>
+      </c>
+      <c r="E1642" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1642" s="4" t="s">
+        <v>3409</v>
+      </c>
+      <c r="G1642" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1642" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="I1642" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1642" s="4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="K1642" s="4" t="s">
+        <v>3440</v>
+      </c>
+      <c r="L1642" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1642" s="4" t="s">
+        <v>2506</v>
+      </c>
+    </row>
+    <row r="1643" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1643" s="4">
+        <v>664</v>
+      </c>
+      <c r="B1643" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1643" s="4">
+        <v>62155</v>
+      </c>
+      <c r="D1643" s="2">
+        <v>46304</v>
+      </c>
+      <c r="E1643" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1643" s="4" t="s">
+        <v>3410</v>
+      </c>
+      <c r="G1643" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1643" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="I1643" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1643" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1643" s="4" t="s">
+        <v>3441</v>
+      </c>
+      <c r="L1643" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1643" s="4" t="s">
+        <v>2534</v>
+      </c>
+    </row>
+    <row r="1644" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1644" s="4">
+        <v>665</v>
+      </c>
+      <c r="B1644" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1644" s="4">
+        <v>151848</v>
+      </c>
+      <c r="D1644" s="2">
+        <v>46305</v>
+      </c>
+      <c r="E1644" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1644" s="4" t="s">
+        <v>3411</v>
+      </c>
+      <c r="G1644" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1644" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1644" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1644" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1644" s="4" t="s">
+        <v>3442</v>
+      </c>
+      <c r="L1644" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1644" s="4" t="s">
+        <v>2413</v>
+      </c>
+    </row>
+    <row r="1645" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1645" s="4">
+        <v>666</v>
+      </c>
+      <c r="B1645" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1645" s="4">
+        <v>154245</v>
+      </c>
+      <c r="D1645" s="2">
+        <v>46305</v>
+      </c>
+      <c r="E1645" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1645" s="4" t="s">
+        <v>3412</v>
+      </c>
+      <c r="G1645" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1645" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1645" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1645" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1645" s="4" t="s">
+        <v>3443</v>
+      </c>
+      <c r="L1645" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1645" s="4" t="s">
+        <v>2413</v>
+      </c>
+    </row>
+    <row r="1646" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1646" s="4">
+        <v>667</v>
+      </c>
+      <c r="B1646" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1646" s="4">
+        <v>158163</v>
+      </c>
+      <c r="D1646" s="2">
+        <v>46305</v>
+      </c>
+      <c r="E1646" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1646" s="4" t="s">
+        <v>3413</v>
+      </c>
+      <c r="G1646" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1646" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="I1646" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1646" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1646" s="4" t="s">
+        <v>3444</v>
+      </c>
+      <c r="L1646" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1646" s="4" t="s">
+        <v>2413</v>
+      </c>
+    </row>
+    <row r="1647" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1647" s="4">
+        <v>668</v>
+      </c>
+      <c r="B1647" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1647" s="4">
+        <v>65384</v>
+      </c>
+      <c r="D1647" s="2">
+        <v>46305</v>
+      </c>
+      <c r="E1647" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1647" s="4" t="s">
+        <v>3414</v>
+      </c>
+      <c r="G1647" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1647" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1647" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1647" s="4" t="s">
+        <v>1359</v>
+      </c>
+      <c r="K1647" s="4" t="s">
+        <v>3445</v>
+      </c>
+      <c r="L1647" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1647" s="4" t="s">
+        <v>2534</v>
+      </c>
+    </row>
+    <row r="1648" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1648" s="4">
+        <v>669</v>
+      </c>
+      <c r="B1648" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1648" s="4">
+        <v>161441</v>
+      </c>
+      <c r="D1648" s="2">
+        <v>46306</v>
+      </c>
+      <c r="E1648" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1648" s="4" t="s">
+        <v>3415</v>
+      </c>
+      <c r="G1648" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1648" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1648" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1648" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1648" s="4" t="s">
+        <v>3446</v>
+      </c>
+      <c r="L1648" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1648" s="4" t="s">
+        <v>2488</v>
+      </c>
+    </row>
+    <row r="1649" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1649" s="4">
+        <v>670</v>
+      </c>
+      <c r="B1649" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1649" s="4">
+        <v>162410</v>
+      </c>
+      <c r="D1649" s="2">
+        <v>46307</v>
+      </c>
+      <c r="E1649" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1649" s="4" t="s">
+        <v>3416</v>
+      </c>
+      <c r="G1649" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1649" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1649" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1649" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1649" s="4" t="s">
+        <v>3447</v>
+      </c>
+      <c r="L1649" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1649" s="4" t="s">
+        <v>2513</v>
+      </c>
+    </row>
+    <row r="1650" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1650" s="4">
+        <v>671</v>
+      </c>
+      <c r="B1650" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1650" s="4">
+        <v>164338</v>
+      </c>
+      <c r="D1650" s="2">
+        <v>46307</v>
+      </c>
+      <c r="E1650" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1650" s="4" t="s">
+        <v>3417</v>
+      </c>
+      <c r="G1650" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1650" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1650" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1650" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1650" s="4" t="s">
+        <v>3448</v>
+      </c>
+      <c r="L1650" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1650" s="4" t="s">
+        <v>2488</v>
+      </c>
+    </row>
+    <row r="1651" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1651" s="4">
+        <v>672</v>
+      </c>
+      <c r="B1651" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1651" s="4">
+        <v>150983</v>
+      </c>
+      <c r="D1651" s="2">
+        <v>46307</v>
+      </c>
+      <c r="E1651" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1651" s="4" t="s">
+        <v>3418</v>
+      </c>
+      <c r="G1651" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1651" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="I1651" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1651" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1651" s="4" t="s">
+        <v>3449</v>
+      </c>
+      <c r="L1651" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1651" s="4" t="s">
+        <v>2506</v>
+      </c>
+    </row>
+    <row r="1652" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1652" s="4">
+        <v>673</v>
+      </c>
+      <c r="B1652" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1652" s="4">
+        <v>158923</v>
+      </c>
+      <c r="D1652" s="2">
+        <v>46308</v>
+      </c>
+      <c r="E1652" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1652" s="4" t="s">
+        <v>3419</v>
+      </c>
+      <c r="G1652" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1652" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I1652" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1652" s="4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="K1652" s="4" t="s">
+        <v>3450</v>
+      </c>
+      <c r="L1652" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1652" s="4" t="s">
+        <v>2494</v>
+      </c>
+    </row>
+    <row r="1653" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1653" s="4">
+        <v>674</v>
+      </c>
+      <c r="B1653" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1653" s="4">
+        <v>161620</v>
+      </c>
+      <c r="D1653" s="2">
+        <v>46308</v>
+      </c>
+      <c r="E1653" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1653" s="4" t="s">
+        <v>3420</v>
+      </c>
+      <c r="G1653" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1653" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1653" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1653" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1653" s="4" t="s">
+        <v>3451</v>
+      </c>
+      <c r="L1653" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1653" s="4" t="s">
+        <v>2410</v>
+      </c>
+    </row>
+    <row r="1654" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1654" s="4">
+        <v>675</v>
+      </c>
+      <c r="B1654" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1654" s="4">
+        <v>152917</v>
+      </c>
+      <c r="D1654" s="2">
+        <v>46308</v>
+      </c>
+      <c r="E1654" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1654" s="4" t="s">
+        <v>3421</v>
+      </c>
+      <c r="G1654" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1654" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I1654" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1654" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1654" s="4" t="s">
+        <v>3452</v>
+      </c>
+      <c r="L1654" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1654" s="4" t="s">
+        <v>2484</v>
+      </c>
+    </row>
+    <row r="1655" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1655" s="4">
+        <v>676</v>
+      </c>
+      <c r="B1655" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1655" s="4">
+        <v>166349</v>
+      </c>
+      <c r="D1655" s="2">
+        <v>46308</v>
+      </c>
+      <c r="E1655" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1655" s="4" t="s">
+        <v>3422</v>
+      </c>
+      <c r="G1655" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1655" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1655" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1655" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1655" s="4" t="s">
+        <v>3453</v>
+      </c>
+      <c r="L1655" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1655" s="4" t="s">
+        <v>2412</v>
+      </c>
+    </row>
+    <row r="1656" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1656" s="4">
+        <v>677</v>
+      </c>
+      <c r="B1656" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1656" s="4">
+        <v>159125</v>
+      </c>
+      <c r="D1656" s="2">
+        <v>46308</v>
+      </c>
+      <c r="E1656" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1656" s="4" t="s">
+        <v>3423</v>
+      </c>
+      <c r="G1656" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1656" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1656" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1656" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1656" s="4" t="s">
+        <v>3454</v>
+      </c>
+      <c r="L1656" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1656" s="4" t="s">
+        <v>2486</v>
+      </c>
+    </row>
+    <row r="1657" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1657" s="4">
+        <v>678</v>
+      </c>
+      <c r="B1657" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1657" s="4">
+        <v>158303</v>
+      </c>
+      <c r="D1657" s="2">
+        <v>46308</v>
+      </c>
+      <c r="E1657" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1657" s="4" t="s">
+        <v>3424</v>
+      </c>
+      <c r="G1657" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1657" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="I1657" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1657" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1657" s="4" t="s">
+        <v>3455</v>
+      </c>
+      <c r="L1657" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1657" s="4" t="s">
+        <v>2488</v>
+      </c>
+    </row>
+    <row r="1658" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1658" s="4">
+        <v>679</v>
+      </c>
+      <c r="B1658" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1658" s="4">
+        <v>164987</v>
+      </c>
+      <c r="D1658" s="2">
+        <v>46308</v>
+      </c>
+      <c r="E1658" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1658" s="5" t="s">
+        <v>3425</v>
+      </c>
+      <c r="G1658" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1658" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1658" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1658" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1658" s="4" t="s">
+        <v>3456</v>
+      </c>
+      <c r="L1658" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1658" s="4" t="s">
+        <v>2517</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 15/10/2026  9:30:33,16
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2867" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5ADB7116-F99D-4A6D-B1FA-5DE68608FF84}"/>
+  <xr:revisionPtr revIDLastSave="2902" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B672193D-AC02-42EE-B637-71757D2F66C7}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16624" uniqueCount="3459">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16704" uniqueCount="3474">
   <si>
     <t>ID</t>
   </si>
@@ -10518,9 +10518,6 @@
 Frustrante isso ! </t>
   </si>
   <si>
-    <t>campo</t>
-  </si>
-  <si>
     <t>FRQ BRASILIA DF R04</t>
   </si>
   <si>
@@ -10703,6 +10700,58 @@
   </si>
   <si>
     <t>mangueira insuficiente + promessa na venda</t>
+  </si>
+  <si>
+    <t>Meu problema nao foi resolvido. Existe uma mistura de assuntos tecnicos com assuntos financeiros. Enfim estou bem desanimada e provavelmente eu desista do serviço.</t>
+  </si>
+  <si>
+    <t>O processo de agendamento de manutenção tem se mostrado bastante moroso. A Culligan não possui um controle proativo das manutenções, fazendo com que seja necessário um acompanhamento constante da nossa parte para que os agendamentos sejam realizados.
+Hoje foi efetuada a manutenção para troca dos filtros dos bebedouros. No entanto, apesar de possuirmos três equipamentos, foi aberta apenas uma Ordem de Serviço (O.S.), quando o correto seria a abertura de uma O.S. para cada bebedouro atendido.
+Ressalto que não houve qualquer problema em relação ao técnico responsável pelo atendimento. O serviço foi executado de forma adequada, e o profissional demonstrou ser extremamente educado, cordial e prestativo durante toda a manutenção.</t>
+  </si>
+  <si>
+    <t>Apesar das manutenções em dia, um dia saiu uma larva viva junto com a agua. TIve uma dificuldade absurda de marcar direito uma manutenção. No dia que o tecnico veio ele não sabia o que fazer (eu não estava em casa, mas a central DEVERIA TER PASSADO AS INFORMAÇÕES). Que experiência patética.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nao sei ainda se está consertado! Vou aguardar </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Técnico não  reparou o filtro e, além disso, terminou de quebra-lo! Foi embora e me deixou com o filtro quebrado e sem água. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muita demora no atendimento e profissional vai despreparado para fazer possíveis reparos </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não apareceu ninguém para fazer a manutenção, e nossa loja é aberta das 10;00 as 22;00h, todos os dias da semana!!! um verdadeiro descaso por parte de vcs.
+grato! </t>
+  </si>
+  <si>
+    <t>A empresa apresentou problemas no sistema de cobrança e ao invés de comunicar claramente e resolver, foi necessário ligar diversas vezes para resolver.
+Além disso, o agendamento de manutenções e/ou trocas de endereço é sempre ruim.</t>
+  </si>
+  <si>
+    <t>problema não foi resolvido + mistura técnico/financeiro</t>
+  </si>
+  <si>
+    <t>agendamento de manutenção moroso + 1 OS para 3 equipamentos</t>
+  </si>
+  <si>
+    <t>saiu uma larva viva + dificuldade de agendar/técnico sem informação</t>
+  </si>
+  <si>
+    <t>não sei se está consertado</t>
+  </si>
+  <si>
+    <t>terminou de quebrá-lo, fiquei sem água (R5)</t>
+  </si>
+  <si>
+    <t>profissional vai despreparado + muita demora no atendimento</t>
+  </si>
+  <si>
+    <t>não apareceu ninguém para a manutenção</t>
+  </si>
+  <si>
+    <t>problemas no sistema de cobrança + agendamento ruim</t>
   </si>
 </sst>
 </file>
@@ -11158,7 +11207,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1658"/>
+  <dimension ref="A1:M1666"/>
   <sheetFormatPr defaultRowHeight="24" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -77834,7 +77883,7 @@
         <v>1338</v>
       </c>
       <c r="K1626" s="4" t="s">
-        <v>3426</v>
+        <v>3425</v>
       </c>
       <c r="L1626" s="4" t="s">
         <v>1547</v>
@@ -77875,7 +77924,7 @@
         <v>1337</v>
       </c>
       <c r="K1627" s="4" t="s">
-        <v>3427</v>
+        <v>3426</v>
       </c>
       <c r="L1627" s="4" t="s">
         <v>1546</v>
@@ -77916,7 +77965,7 @@
         <v>1337</v>
       </c>
       <c r="K1628" s="4" t="s">
-        <v>3428</v>
+        <v>3427</v>
       </c>
       <c r="L1628" s="4" t="s">
         <v>1547</v>
@@ -77957,7 +78006,7 @@
         <v>1337</v>
       </c>
       <c r="K1629" s="4" t="s">
-        <v>3429</v>
+        <v>3428</v>
       </c>
       <c r="L1629" s="4" t="s">
         <v>1547</v>
@@ -77986,7 +78035,7 @@
         <v>3396</v>
       </c>
       <c r="G1630" s="4" t="s">
-        <v>3401</v>
+        <v>15</v>
       </c>
       <c r="H1630" s="4" t="s">
         <v>40</v>
@@ -77998,7 +78047,7 @@
         <v>1337</v>
       </c>
       <c r="K1630" s="4" t="s">
-        <v>3430</v>
+        <v>3429</v>
       </c>
       <c r="L1630" s="4" t="s">
         <v>1546</v>
@@ -78027,7 +78076,7 @@
         <v>3397</v>
       </c>
       <c r="G1631" s="4" t="s">
-        <v>3401</v>
+        <v>15</v>
       </c>
       <c r="H1631" s="4" t="s">
         <v>18</v>
@@ -78039,7 +78088,7 @@
         <v>1337</v>
       </c>
       <c r="K1631" s="4" t="s">
-        <v>3431</v>
+        <v>3430</v>
       </c>
       <c r="L1631" s="4" t="s">
         <v>1547</v>
@@ -78068,7 +78117,7 @@
         <v>3398</v>
       </c>
       <c r="G1632" s="4" t="s">
-        <v>3401</v>
+        <v>15</v>
       </c>
       <c r="H1632" s="4" t="s">
         <v>948</v>
@@ -78080,7 +78129,7 @@
         <v>1337</v>
       </c>
       <c r="K1632" s="4" t="s">
-        <v>3432</v>
+        <v>3431</v>
       </c>
       <c r="L1632" s="4" t="s">
         <v>1546</v>
@@ -78109,7 +78158,7 @@
         <v>3399</v>
       </c>
       <c r="G1633" s="4" t="s">
-        <v>3401</v>
+        <v>15</v>
       </c>
       <c r="H1633" s="4" t="s">
         <v>18</v>
@@ -78121,7 +78170,7 @@
         <v>1337</v>
       </c>
       <c r="K1633" s="4" t="s">
-        <v>3457</v>
+        <v>3456</v>
       </c>
       <c r="L1633" s="4" t="s">
         <v>1547</v>
@@ -78150,7 +78199,7 @@
         <v>3400</v>
       </c>
       <c r="G1634" s="4" t="s">
-        <v>3401</v>
+        <v>15</v>
       </c>
       <c r="H1634" s="4" t="s">
         <v>48</v>
@@ -78162,7 +78211,7 @@
         <v>1337</v>
       </c>
       <c r="K1634" s="4" t="s">
-        <v>3458</v>
+        <v>3457</v>
       </c>
       <c r="L1634" s="4" t="s">
         <v>1547</v>
@@ -78188,7 +78237,7 @@
         <v>13</v>
       </c>
       <c r="F1635" s="4" t="s">
-        <v>3403</v>
+        <v>3402</v>
       </c>
       <c r="G1635" s="4" t="s">
         <v>25</v>
@@ -78203,7 +78252,7 @@
         <v>1337</v>
       </c>
       <c r="K1635" s="4" t="s">
-        <v>3433</v>
+        <v>3432</v>
       </c>
       <c r="L1635" s="4" t="s">
         <v>1546</v>
@@ -78229,7 +78278,7 @@
         <v>13</v>
       </c>
       <c r="F1636" s="4" t="s">
-        <v>3404</v>
+        <v>3403</v>
       </c>
       <c r="G1636" s="4" t="s">
         <v>15</v>
@@ -78244,7 +78293,7 @@
         <v>1337</v>
       </c>
       <c r="K1636" s="4" t="s">
-        <v>3434</v>
+        <v>3433</v>
       </c>
       <c r="L1636" s="4" t="s">
         <v>1546</v>
@@ -78270,7 +78319,7 @@
         <v>13</v>
       </c>
       <c r="F1637" s="4" t="s">
-        <v>3405</v>
+        <v>3404</v>
       </c>
       <c r="G1637" s="4" t="s">
         <v>15</v>
@@ -78285,7 +78334,7 @@
         <v>1359</v>
       </c>
       <c r="K1637" s="4" t="s">
-        <v>3435</v>
+        <v>3434</v>
       </c>
       <c r="L1637" s="4" t="s">
         <v>1546</v>
@@ -78311,7 +78360,7 @@
         <v>13</v>
       </c>
       <c r="F1638" s="4" t="s">
-        <v>3406</v>
+        <v>3405</v>
       </c>
       <c r="G1638" s="4" t="s">
         <v>3394</v>
@@ -78326,7 +78375,7 @@
         <v>1337</v>
       </c>
       <c r="K1638" s="4" t="s">
-        <v>3436</v>
+        <v>3435</v>
       </c>
       <c r="L1638" s="4" t="s">
         <v>1546</v>
@@ -78352,7 +78401,7 @@
         <v>13</v>
       </c>
       <c r="F1639" s="4" t="s">
-        <v>3407</v>
+        <v>3406</v>
       </c>
       <c r="G1639" s="4" t="s">
         <v>25</v>
@@ -78367,7 +78416,7 @@
         <v>1337</v>
       </c>
       <c r="K1639" s="4" t="s">
-        <v>3437</v>
+        <v>3436</v>
       </c>
       <c r="L1639" s="4" t="s">
         <v>1546</v>
@@ -78393,7 +78442,7 @@
         <v>13</v>
       </c>
       <c r="F1640" s="4" t="s">
-        <v>3408</v>
+        <v>3407</v>
       </c>
       <c r="G1640" s="4" t="s">
         <v>25</v>
@@ -78408,13 +78457,13 @@
         <v>1337</v>
       </c>
       <c r="K1640" s="4" t="s">
-        <v>3438</v>
+        <v>3437</v>
       </c>
       <c r="L1640" s="4" t="s">
         <v>1546</v>
       </c>
       <c r="M1640" s="4" t="s">
-        <v>3402</v>
+        <v>3401</v>
       </c>
     </row>
     <row r="1641" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -78449,7 +78498,7 @@
         <v>1337</v>
       </c>
       <c r="K1641" s="4" t="s">
-        <v>3439</v>
+        <v>3438</v>
       </c>
       <c r="L1641" s="4" t="s">
         <v>1547</v>
@@ -78475,7 +78524,7 @@
         <v>13</v>
       </c>
       <c r="F1642" s="4" t="s">
-        <v>3409</v>
+        <v>3408</v>
       </c>
       <c r="G1642" s="4" t="s">
         <v>28</v>
@@ -78490,7 +78539,7 @@
         <v>1338</v>
       </c>
       <c r="K1642" s="4" t="s">
-        <v>3440</v>
+        <v>3439</v>
       </c>
       <c r="L1642" s="4" t="s">
         <v>1546</v>
@@ -78516,7 +78565,7 @@
         <v>13</v>
       </c>
       <c r="F1643" s="4" t="s">
-        <v>3410</v>
+        <v>3409</v>
       </c>
       <c r="G1643" s="4" t="s">
         <v>65</v>
@@ -78531,7 +78580,7 @@
         <v>1337</v>
       </c>
       <c r="K1643" s="4" t="s">
-        <v>3441</v>
+        <v>3440</v>
       </c>
       <c r="L1643" s="4" t="s">
         <v>1546</v>
@@ -78557,7 +78606,7 @@
         <v>13</v>
       </c>
       <c r="F1644" s="4" t="s">
-        <v>3411</v>
+        <v>3410</v>
       </c>
       <c r="G1644" s="4" t="s">
         <v>15</v>
@@ -78572,7 +78621,7 @@
         <v>1337</v>
       </c>
       <c r="K1644" s="4" t="s">
-        <v>3442</v>
+        <v>3441</v>
       </c>
       <c r="L1644" s="4" t="s">
         <v>1547</v>
@@ -78598,7 +78647,7 @@
         <v>13</v>
       </c>
       <c r="F1645" s="4" t="s">
-        <v>3412</v>
+        <v>3411</v>
       </c>
       <c r="G1645" s="4" t="s">
         <v>15</v>
@@ -78613,7 +78662,7 @@
         <v>1337</v>
       </c>
       <c r="K1645" s="4" t="s">
-        <v>3443</v>
+        <v>3442</v>
       </c>
       <c r="L1645" s="4" t="s">
         <v>1547</v>
@@ -78639,7 +78688,7 @@
         <v>13</v>
       </c>
       <c r="F1646" s="4" t="s">
-        <v>3413</v>
+        <v>3412</v>
       </c>
       <c r="G1646" s="4" t="s">
         <v>65</v>
@@ -78654,7 +78703,7 @@
         <v>1337</v>
       </c>
       <c r="K1646" s="4" t="s">
-        <v>3444</v>
+        <v>3443</v>
       </c>
       <c r="L1646" s="4" t="s">
         <v>1547</v>
@@ -78680,7 +78729,7 @@
         <v>13</v>
       </c>
       <c r="F1647" s="4" t="s">
-        <v>3414</v>
+        <v>3413</v>
       </c>
       <c r="G1647" s="4" t="s">
         <v>15</v>
@@ -78695,7 +78744,7 @@
         <v>1359</v>
       </c>
       <c r="K1647" s="4" t="s">
-        <v>3445</v>
+        <v>3444</v>
       </c>
       <c r="L1647" s="4" t="s">
         <v>1546</v>
@@ -78721,7 +78770,7 @@
         <v>13</v>
       </c>
       <c r="F1648" s="4" t="s">
-        <v>3415</v>
+        <v>3414</v>
       </c>
       <c r="G1648" s="4" t="s">
         <v>15</v>
@@ -78736,7 +78785,7 @@
         <v>1337</v>
       </c>
       <c r="K1648" s="4" t="s">
-        <v>3446</v>
+        <v>3445</v>
       </c>
       <c r="L1648" s="4" t="s">
         <v>1546</v>
@@ -78762,7 +78811,7 @@
         <v>13</v>
       </c>
       <c r="F1649" s="4" t="s">
-        <v>3416</v>
+        <v>3415</v>
       </c>
       <c r="G1649" s="4" t="s">
         <v>15</v>
@@ -78777,7 +78826,7 @@
         <v>1337</v>
       </c>
       <c r="K1649" s="4" t="s">
-        <v>3447</v>
+        <v>3446</v>
       </c>
       <c r="L1649" s="4" t="s">
         <v>1546</v>
@@ -78803,7 +78852,7 @@
         <v>13</v>
       </c>
       <c r="F1650" s="4" t="s">
-        <v>3417</v>
+        <v>3416</v>
       </c>
       <c r="G1650" s="4" t="s">
         <v>15</v>
@@ -78818,7 +78867,7 @@
         <v>1337</v>
       </c>
       <c r="K1650" s="4" t="s">
-        <v>3448</v>
+        <v>3447</v>
       </c>
       <c r="L1650" s="4" t="s">
         <v>1546</v>
@@ -78844,7 +78893,7 @@
         <v>13</v>
       </c>
       <c r="F1651" s="4" t="s">
-        <v>3418</v>
+        <v>3417</v>
       </c>
       <c r="G1651" s="4" t="s">
         <v>28</v>
@@ -78859,7 +78908,7 @@
         <v>1337</v>
       </c>
       <c r="K1651" s="4" t="s">
-        <v>3449</v>
+        <v>3448</v>
       </c>
       <c r="L1651" s="4" t="s">
         <v>1546</v>
@@ -78885,7 +78934,7 @@
         <v>13</v>
       </c>
       <c r="F1652" s="4" t="s">
-        <v>3419</v>
+        <v>3418</v>
       </c>
       <c r="G1652" s="4" t="s">
         <v>15</v>
@@ -78900,7 +78949,7 @@
         <v>1338</v>
       </c>
       <c r="K1652" s="4" t="s">
-        <v>3450</v>
+        <v>3449</v>
       </c>
       <c r="L1652" s="4" t="s">
         <v>1546</v>
@@ -78926,7 +78975,7 @@
         <v>13</v>
       </c>
       <c r="F1653" s="4" t="s">
-        <v>3420</v>
+        <v>3419</v>
       </c>
       <c r="G1653" s="4" t="s">
         <v>15</v>
@@ -78941,7 +78990,7 @@
         <v>1337</v>
       </c>
       <c r="K1653" s="4" t="s">
-        <v>3451</v>
+        <v>3450</v>
       </c>
       <c r="L1653" s="4" t="s">
         <v>1546</v>
@@ -78967,7 +79016,7 @@
         <v>13</v>
       </c>
       <c r="F1654" s="4" t="s">
-        <v>3421</v>
+        <v>3420</v>
       </c>
       <c r="G1654" s="4" t="s">
         <v>15</v>
@@ -78982,7 +79031,7 @@
         <v>1337</v>
       </c>
       <c r="K1654" s="4" t="s">
-        <v>3452</v>
+        <v>3451</v>
       </c>
       <c r="L1654" s="4" t="s">
         <v>1546</v>
@@ -79008,7 +79057,7 @@
         <v>13</v>
       </c>
       <c r="F1655" s="4" t="s">
-        <v>3422</v>
+        <v>3421</v>
       </c>
       <c r="G1655" s="4" t="s">
         <v>15</v>
@@ -79023,7 +79072,7 @@
         <v>1337</v>
       </c>
       <c r="K1655" s="4" t="s">
-        <v>3453</v>
+        <v>3452</v>
       </c>
       <c r="L1655" s="4" t="s">
         <v>1546</v>
@@ -79049,7 +79098,7 @@
         <v>13</v>
       </c>
       <c r="F1656" s="4" t="s">
-        <v>3423</v>
+        <v>3422</v>
       </c>
       <c r="G1656" s="4" t="s">
         <v>15</v>
@@ -79064,7 +79113,7 @@
         <v>1337</v>
       </c>
       <c r="K1656" s="4" t="s">
-        <v>3454</v>
+        <v>3453</v>
       </c>
       <c r="L1656" s="4" t="s">
         <v>1547</v>
@@ -79090,7 +79139,7 @@
         <v>13</v>
       </c>
       <c r="F1657" s="4" t="s">
-        <v>3424</v>
+        <v>3423</v>
       </c>
       <c r="G1657" s="4" t="s">
         <v>28</v>
@@ -79105,7 +79154,7 @@
         <v>1337</v>
       </c>
       <c r="K1657" s="4" t="s">
-        <v>3455</v>
+        <v>3454</v>
       </c>
       <c r="L1657" s="4" t="s">
         <v>1547</v>
@@ -79131,7 +79180,7 @@
         <v>13</v>
       </c>
       <c r="F1658" s="5" t="s">
-        <v>3425</v>
+        <v>3424</v>
       </c>
       <c r="G1658" s="4" t="s">
         <v>28</v>
@@ -79146,13 +79195,341 @@
         <v>1337</v>
       </c>
       <c r="K1658" s="4" t="s">
-        <v>3456</v>
+        <v>3455</v>
       </c>
       <c r="L1658" s="4" t="s">
         <v>1546</v>
       </c>
       <c r="M1658" s="4" t="s">
         <v>2517</v>
+      </c>
+    </row>
+    <row r="1659" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1659" s="4">
+        <v>680</v>
+      </c>
+      <c r="B1659" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1659" s="4">
+        <v>155845</v>
+      </c>
+      <c r="D1659" s="2">
+        <v>46309</v>
+      </c>
+      <c r="E1659" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1659" s="4" t="s">
+        <v>3458</v>
+      </c>
+      <c r="G1659" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1659" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1659" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1659" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1659" s="4" t="s">
+        <v>3466</v>
+      </c>
+      <c r="L1659" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1659" s="4" t="s">
+        <v>2447</v>
+      </c>
+    </row>
+    <row r="1660" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1660" s="4">
+        <v>681</v>
+      </c>
+      <c r="B1660" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1660" s="4">
+        <v>143350</v>
+      </c>
+      <c r="D1660" s="2">
+        <v>46309</v>
+      </c>
+      <c r="E1660" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1660" s="5" t="s">
+        <v>3459</v>
+      </c>
+      <c r="G1660" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1660" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1660" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1660" s="4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="K1660" s="4" t="s">
+        <v>3467</v>
+      </c>
+      <c r="L1660" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1660" s="4" t="s">
+        <v>2532</v>
+      </c>
+    </row>
+    <row r="1661" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1661" s="4">
+        <v>682</v>
+      </c>
+      <c r="B1661" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1661" s="4">
+        <v>166438</v>
+      </c>
+      <c r="D1661" s="2">
+        <v>46309</v>
+      </c>
+      <c r="E1661" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1661" s="4" t="s">
+        <v>3460</v>
+      </c>
+      <c r="G1661" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1661" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="I1661" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1661" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1661" s="4" t="s">
+        <v>3468</v>
+      </c>
+      <c r="L1661" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1661" s="4" t="s">
+        <v>2494</v>
+      </c>
+    </row>
+    <row r="1662" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1662" s="4">
+        <v>683</v>
+      </c>
+      <c r="B1662" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1662" s="4">
+        <v>166797</v>
+      </c>
+      <c r="D1662" s="2">
+        <v>46309</v>
+      </c>
+      <c r="E1662" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1662" s="4" t="s">
+        <v>3461</v>
+      </c>
+      <c r="G1662" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1662" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1662" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1662" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1662" s="4" t="s">
+        <v>3469</v>
+      </c>
+      <c r="L1662" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1662" s="4" t="s">
+        <v>2494</v>
+      </c>
+    </row>
+    <row r="1663" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1663" s="4">
+        <v>684</v>
+      </c>
+      <c r="B1663" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1663" s="4">
+        <v>166156</v>
+      </c>
+      <c r="D1663" s="2">
+        <v>46309</v>
+      </c>
+      <c r="E1663" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1663" s="4" t="s">
+        <v>3462</v>
+      </c>
+      <c r="G1663" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1663" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I1663" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1663" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1663" s="4" t="s">
+        <v>3470</v>
+      </c>
+      <c r="L1663" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1663" s="4" t="s">
+        <v>2494</v>
+      </c>
+    </row>
+    <row r="1664" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1664" s="4">
+        <v>685</v>
+      </c>
+      <c r="B1664" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1664" s="4">
+        <v>166940</v>
+      </c>
+      <c r="D1664" s="2">
+        <v>46309</v>
+      </c>
+      <c r="E1664" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1664" s="4" t="s">
+        <v>3463</v>
+      </c>
+      <c r="G1664" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1664" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I1664" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1664" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1664" s="4" t="s">
+        <v>3471</v>
+      </c>
+      <c r="L1664" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1664" s="4" t="s">
+        <v>2508</v>
+      </c>
+    </row>
+    <row r="1665" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1665" s="4">
+        <v>686</v>
+      </c>
+      <c r="B1665" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1665" s="4">
+        <v>155765</v>
+      </c>
+      <c r="D1665" s="2">
+        <v>46309</v>
+      </c>
+      <c r="E1665" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1665" s="4" t="s">
+        <v>3464</v>
+      </c>
+      <c r="G1665" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1665" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1665" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1665" s="4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="K1665" s="4" t="s">
+        <v>3472</v>
+      </c>
+      <c r="L1665" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1665" s="4" t="s">
+        <v>2412</v>
+      </c>
+    </row>
+    <row r="1666" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1666" s="4">
+        <v>687</v>
+      </c>
+      <c r="B1666" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1666" s="4">
+        <v>157572</v>
+      </c>
+      <c r="D1666" s="2">
+        <v>46310</v>
+      </c>
+      <c r="E1666" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1666" s="4" t="s">
+        <v>3465</v>
+      </c>
+      <c r="G1666" s="4" t="s">
+        <v>3394</v>
+      </c>
+      <c r="H1666" s="4" t="s">
+        <v>3395</v>
+      </c>
+      <c r="I1666" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1666" s="4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="K1666" s="4" t="s">
+        <v>3473</v>
+      </c>
+      <c r="L1666" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1666" s="4" t="s">
+        <v>2446</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 16/10/2026 11:38:23,38
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2902" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B672193D-AC02-42EE-B637-71757D2F66C7}"/>
+  <xr:revisionPtr revIDLastSave="2940" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2BED1B3-627B-41E7-8003-DCC1C8FA535B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16704" uniqueCount="3474">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16764" uniqueCount="3487">
   <si>
     <t>ID</t>
   </si>
@@ -10752,6 +10752,48 @@
   </si>
   <si>
     <t>problemas no sistema de cobrança + agendamento ruim</t>
+  </si>
+  <si>
+    <t>Lixo de serviço!!! Não monitoram o tempo das manutenções periódicas e não respondem ao canal oficial de WhatsApp da própria empresa!!! Jamais recomendarei a alguém.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">So um técnico realmente limpou tudo, a fan as aletas de entrada de ar. Os atuais so passam um pano por fora e um cotonete.  Isso eu ja faço por higiene. </t>
+  </si>
+  <si>
+    <t>Porque o cliente marca o horário de atendimento pela manhã de 8:00 às 13:00 e no entanto o técnico só chegou às 14:30 h.
+Ou seja atrapalha a vida do cliente.
+E a culpa é da empresa que faz um itinerário errado do técnico pois marca mais clientes do que deve.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pq fiquei 1 ano sem a visita técnica,ligo para pedir uma visita e marquei por 3 vezes e as 3 vezes marcadas a visita,não foram nenhuma, alegam sempre alguma coisa, os contatos com a empresa e péssimo um robô que nunca quase deixa vc ter um contato para maior esclarecimento e sempre terminando a conversa,e o pior com dois representantes o de são Paulo e do Rio de janeiro,que não se entendem e o robô marcando a visita técnica e cancelando uma verdadeira bagunça no qual ninguém se entende. </t>
+  </si>
+  <si>
+    <t>Fiz o upgrade para um novo plano. Porém me trouxerem o mesmo purificador do plano antigo.</t>
+  </si>
+  <si>
+    <t>Não tive visita do técnico pois ficou agendado para parte da tarde e o mesmo chegou às 11:05 hs e eu estava na rua pois o agendamento começava às 13 hs.
+Uma vergonha !</t>
+  </si>
+  <si>
+    <t>AT SJRPRETO SP R04</t>
+  </si>
+  <si>
+    <t>não monitoram manutenções periódicas + WhatsApp não responde</t>
+  </si>
+  <si>
+    <t>só passam um pano por fora</t>
+  </si>
+  <si>
+    <t>marcado 8h-13h, técnico chegou 14:30</t>
+  </si>
+  <si>
+    <t>3 visitas marcadas, nenhuma ocorreu + contato via robô péssimo</t>
+  </si>
+  <si>
+    <t>upgrade, mas trouxeram mesmo purificador antigo</t>
+  </si>
+  <si>
+    <t>agendado à tarde, chegou às 11:05</t>
   </si>
 </sst>
 </file>
@@ -11207,7 +11249,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1666"/>
+  <dimension ref="A1:M1672"/>
   <sheetFormatPr defaultRowHeight="24" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -79532,6 +79574,252 @@
         <v>2446</v>
       </c>
     </row>
+    <row r="1667" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1667" s="4">
+        <v>688</v>
+      </c>
+      <c r="B1667" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1667" s="4">
+        <v>155583</v>
+      </c>
+      <c r="D1667" s="2">
+        <v>46310</v>
+      </c>
+      <c r="E1667" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1667" s="4" t="s">
+        <v>3474</v>
+      </c>
+      <c r="G1667" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1667" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="I1667" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1667" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1667" s="4" t="s">
+        <v>3481</v>
+      </c>
+      <c r="L1667" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1667" s="4" t="s">
+        <v>2487</v>
+      </c>
+    </row>
+    <row r="1668" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1668" s="4">
+        <v>689</v>
+      </c>
+      <c r="B1668" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1668" s="4">
+        <v>163783</v>
+      </c>
+      <c r="D1668" s="2">
+        <v>46310</v>
+      </c>
+      <c r="E1668" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1668" s="4" t="s">
+        <v>3475</v>
+      </c>
+      <c r="G1668" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1668" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I1668" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1668" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1668" s="4" t="s">
+        <v>3482</v>
+      </c>
+      <c r="L1668" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1668" s="4" t="s">
+        <v>2506</v>
+      </c>
+    </row>
+    <row r="1669" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1669" s="4">
+        <v>690</v>
+      </c>
+      <c r="B1669" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1669" s="4">
+        <v>151864</v>
+      </c>
+      <c r="D1669" s="2">
+        <v>46310</v>
+      </c>
+      <c r="E1669" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1669" s="4" t="s">
+        <v>3476</v>
+      </c>
+      <c r="G1669" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1669" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1669" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1669" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1669" s="4" t="s">
+        <v>3483</v>
+      </c>
+      <c r="L1669" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1669" s="4" t="s">
+        <v>2410</v>
+      </c>
+    </row>
+    <row r="1670" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1670" s="4">
+        <v>691</v>
+      </c>
+      <c r="B1670" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1670" s="4">
+        <v>169636</v>
+      </c>
+      <c r="D1670" s="2">
+        <v>46310</v>
+      </c>
+      <c r="E1670" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1670" s="4" t="s">
+        <v>3477</v>
+      </c>
+      <c r="G1670" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1670" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1670" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1670" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1670" s="4" t="s">
+        <v>3484</v>
+      </c>
+      <c r="L1670" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1670" s="4" t="s">
+        <v>2484</v>
+      </c>
+    </row>
+    <row r="1671" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1671" s="4">
+        <v>692</v>
+      </c>
+      <c r="B1671" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1671" s="4">
+        <v>167755</v>
+      </c>
+      <c r="D1671" s="2">
+        <v>46310</v>
+      </c>
+      <c r="E1671" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1671" s="4" t="s">
+        <v>3478</v>
+      </c>
+      <c r="G1671" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1671" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1671" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1671" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1671" s="4" t="s">
+        <v>3485</v>
+      </c>
+      <c r="L1671" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1671" s="4" t="s">
+        <v>3480</v>
+      </c>
+    </row>
+    <row r="1672" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1672" s="4">
+        <v>693</v>
+      </c>
+      <c r="B1672" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1672" s="4">
+        <v>157462</v>
+      </c>
+      <c r="D1672" s="2">
+        <v>46310</v>
+      </c>
+      <c r="E1672" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1672" s="4" t="s">
+        <v>3479</v>
+      </c>
+      <c r="G1672" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1672" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1672" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1672" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1672" s="4" t="s">
+        <v>3486</v>
+      </c>
+      <c r="L1672" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1672" s="4" t="s">
+        <v>2488</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 19/10/2026  9:53:51,05
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2940" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2BED1B3-627B-41E7-8003-DCC1C8FA535B}"/>
+  <xr:revisionPtr revIDLastSave="2955" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02DA56A3-3853-43B1-AE85-B4F681C41140}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16764" uniqueCount="3487">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16788" uniqueCount="3490">
   <si>
     <t>ID</t>
   </si>
@@ -10794,6 +10794,15 @@
   </si>
   <si>
     <t>agendado à tarde, chegou às 11:05</t>
+  </si>
+  <si>
+    <t>Nao compareceram para trocar o filtro que veio errado</t>
+  </si>
+  <si>
+    <t>Atendimento péssimo, gostaria que vocês escutassem a gravação das minhas ligações</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Porque existem no mercado filtros de qualidade por um preço muito bom </t>
   </si>
 </sst>
 </file>
@@ -11249,7 +11258,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1672"/>
+  <dimension ref="A1:M1675"/>
   <sheetFormatPr defaultRowHeight="24" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -79820,6 +79829,111 @@
         <v>2488</v>
       </c>
     </row>
+    <row r="1673" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1673" s="4">
+        <v>694</v>
+      </c>
+      <c r="B1673" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1673" s="4">
+        <v>162322</v>
+      </c>
+      <c r="D1673" s="2">
+        <v>46311</v>
+      </c>
+      <c r="E1673" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1673" s="4" t="s">
+        <v>3487</v>
+      </c>
+      <c r="G1673" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1673" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1673" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1673" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1673" s="4" t="s">
+        <v>2446</v>
+      </c>
+    </row>
+    <row r="1674" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1674" s="4">
+        <v>695</v>
+      </c>
+      <c r="B1674" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1674" s="4">
+        <v>158327</v>
+      </c>
+      <c r="D1674" s="2">
+        <v>46311</v>
+      </c>
+      <c r="E1674" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1674" s="4" t="s">
+        <v>3488</v>
+      </c>
+      <c r="G1674" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1674" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="I1674" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1674" s="4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="M1674" s="4" t="s">
+        <v>2515</v>
+      </c>
+    </row>
+    <row r="1675" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1675" s="4">
+        <v>696</v>
+      </c>
+      <c r="B1675" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1675" s="4">
+        <v>150676</v>
+      </c>
+      <c r="D1675" s="2">
+        <v>46312</v>
+      </c>
+      <c r="E1675" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1675" s="4" t="s">
+        <v>3489</v>
+      </c>
+      <c r="G1675" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1675" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="I1675" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1675" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="M1675" s="4" t="s">
+        <v>2410</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 21/10/2026  8:19:57,77
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2955" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02DA56A3-3853-43B1-AE85-B4F681C41140}"/>
+  <xr:revisionPtr revIDLastSave="2985" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97CF54E0-1014-43C5-A229-BF0758F4691B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16788" uniqueCount="3490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16842" uniqueCount="3500">
   <si>
     <t>ID</t>
   </si>
@@ -10803,6 +10803,39 @@
   </si>
   <si>
     <t xml:space="preserve">Porque existem no mercado filtros de qualidade por um preço muito bom </t>
+  </si>
+  <si>
+    <t>Continuam com péssimo atendimento e relacionamento. Estou aguardando há 4 anos solução… Ainda está tudo muito confuso… não sei até onde vou continuar com vocês… a insatisfação é grande…</t>
+  </si>
+  <si>
+    <t>A CLASSIFICAÇÃO FOI BAIXA DEVIDO QUE PRECISAVAMOS RESOLVER O PROBLEMA, E NO FINAL TEREMOS QUE FICAR SEM AGUA POR 24 HORAS, TRABALHAMOS COM O PUBLICO. E ALEM DE TUDO ESTÁ UM DIA SUPER QUENTE.</t>
+  </si>
+  <si>
+    <t>já agendei visita técnica para reparos pela terceira vez e , nenhum técnico apareceu até agora
+cnpj 58669565000146 - lofer restaurante - avenida coronel silva teles, 514 - cambui - campinas - FILTRO INSTALADO NO BAR DO SALÃO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Técnico chegou antes das 13h e eu não estava em casa. Retornou as 13h mal-humorado dizendo que a frequência de troca do filtro é de 12 meses e não 6. Não quis ver como a vazão da água havia diminuído e como o elemento estava sujo. Acabou trocando depois que reclamei. Não fez higienização nem nada mais. Não deixou o canhoto do serviço executado comigo. </t>
+  </si>
+  <si>
+    <t>Faltaram para manutenção  preventiva  marcada  para hoje</t>
+  </si>
+  <si>
+    <t>Porque houve demora para o atendimento. Chamado aberto no dia 14/10 e a atendente agendou para somente 22/10 (8 dias depois), mesmo explicando que havia somente um bebedouro no andar para os clientes e de que a clínica abre inclusive nos sábados e domingos.
+Após ligações (que demoram para atender) e emails enviados, suplicando atendimento, é que fomos atendidos no dia 20/10 (6 dias depois).
+Solicitamos desconto dos dias de equipamento parado conforme previsto na cláusula 4.3 do contrato.</t>
+  </si>
+  <si>
+    <t>Eduarda Cândida Jacinta dos Reis</t>
+  </si>
+  <si>
+    <t>Integração BOOMI</t>
+  </si>
+  <si>
+    <t>AlCIONE APARECIDA DE OLIVEIRA</t>
+  </si>
+  <si>
+    <t>Roberta Duarte De Souza</t>
   </si>
 </sst>
 </file>
@@ -11258,7 +11291,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1675"/>
+  <dimension ref="A1:M1681"/>
   <sheetFormatPr defaultRowHeight="24" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -79934,6 +79967,234 @@
         <v>2410</v>
       </c>
     </row>
+    <row r="1676" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1676" s="4">
+        <v>697</v>
+      </c>
+      <c r="B1676" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1676" s="4">
+        <v>165349</v>
+      </c>
+      <c r="D1676" s="2">
+        <v>46315</v>
+      </c>
+      <c r="E1676" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1676" s="4" t="s">
+        <v>3490</v>
+      </c>
+      <c r="G1676" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1676" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1676" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1676" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1676" s="4" t="s">
+        <v>3496</v>
+      </c>
+      <c r="M1676" s="4" t="s">
+        <v>2520</v>
+      </c>
+    </row>
+    <row r="1677" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1677" s="4">
+        <v>698</v>
+      </c>
+      <c r="B1677" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1677" s="4">
+        <v>167550</v>
+      </c>
+      <c r="D1677" s="2">
+        <v>46315</v>
+      </c>
+      <c r="E1677" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1677" s="4" t="s">
+        <v>3491</v>
+      </c>
+      <c r="G1677" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1677" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1677" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1677" s="4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="K1677" s="4" t="s">
+        <v>3497</v>
+      </c>
+      <c r="M1677" s="4" t="s">
+        <v>2527</v>
+      </c>
+    </row>
+    <row r="1678" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1678" s="4">
+        <v>700</v>
+      </c>
+      <c r="B1678" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1678" s="4">
+        <v>167806</v>
+      </c>
+      <c r="D1678" s="2">
+        <v>46315</v>
+      </c>
+      <c r="E1678" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1678" s="5" t="s">
+        <v>3492</v>
+      </c>
+      <c r="G1678" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1678" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1678" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1678" s="4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="K1678" s="4" t="s">
+        <v>3497</v>
+      </c>
+      <c r="M1678" s="4" t="s">
+        <v>2506</v>
+      </c>
+    </row>
+    <row r="1679" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1679" s="4">
+        <v>701</v>
+      </c>
+      <c r="B1679" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1679" s="4">
+        <v>164009</v>
+      </c>
+      <c r="D1679" s="2">
+        <v>46315</v>
+      </c>
+      <c r="E1679" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1679" s="4" t="s">
+        <v>3493</v>
+      </c>
+      <c r="G1679" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1679" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I1679" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1679" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1679" s="4" t="s">
+        <v>3497</v>
+      </c>
+      <c r="M1679" s="4" t="s">
+        <v>2410</v>
+      </c>
+    </row>
+    <row r="1680" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1680" s="4">
+        <v>702</v>
+      </c>
+      <c r="B1680" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C1680" s="4">
+        <v>159120</v>
+      </c>
+      <c r="D1680" s="2">
+        <v>46315</v>
+      </c>
+      <c r="E1680" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1680" s="4" t="s">
+        <v>3494</v>
+      </c>
+      <c r="G1680" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1680" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1680" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1680" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1680" s="4" t="s">
+        <v>3498</v>
+      </c>
+      <c r="M1680" s="4" t="s">
+        <v>2484</v>
+      </c>
+    </row>
+    <row r="1681" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1681" s="4">
+        <v>703</v>
+      </c>
+      <c r="B1681" s="4" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1681" s="4">
+        <v>168842</v>
+      </c>
+      <c r="D1681" s="2">
+        <v>46315</v>
+      </c>
+      <c r="E1681" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1681" s="4" t="s">
+        <v>3495</v>
+      </c>
+      <c r="G1681" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1681" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1681" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1681" s="4" t="s">
+        <v>1359</v>
+      </c>
+      <c r="K1681" s="4" t="s">
+        <v>3499</v>
+      </c>
+      <c r="M1681" s="4" t="s">
+        <v>2534</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Atualizacao de arquivos - 27/10/2026 12:57:34,25
</commit_message>
<xml_diff>
--- a/NPS Classificado.xlsx
+++ b/NPS Classificado.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/eduardacjr_callink_com_br/Documents/Área de Trabalho/Dashboards/nps-franquias/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://callinkcombr-my.sharepoint.com/personal/pedroofs_callink_com_br/Documents/Área de Trabalho/Dashboards/12 - NPS/nps-franquias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3026" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B48BC65-184F-4DFD-9821-732EAB2B5454}"/>
+  <xr:revisionPtr revIDLastSave="3039" documentId="8_{855DE731-06B6-4F67-B5F3-79AE1FB3CA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{827C5AB5-5BBE-41AB-9394-4FA7382F0DC5}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-24120" yWindow="-2580" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16854" uniqueCount="3508">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17206" uniqueCount="3581">
   <si>
     <t>ID</t>
   </si>
@@ -10860,6 +10860,232 @@
   </si>
   <si>
     <t>sem comunicado de agendamento (Large) + unificar preventiva dos 3</t>
+  </si>
+  <si>
+    <t>21/10/2026</t>
+  </si>
+  <si>
+    <t>22/10/2026</t>
+  </si>
+  <si>
+    <t>23/10/2026</t>
+  </si>
+  <si>
+    <t>24/10/2026</t>
+  </si>
+  <si>
+    <t>26/10/2026</t>
+  </si>
+  <si>
+    <t>27/10/2026</t>
+  </si>
+  <si>
+    <t>PORQUE? O TECNICO VEIO NAO ARRUMOU MEU PURIFICADOR, DEPOIS DE ESPERAR MAIS DE UMA SEMANA, E ESSE MÉTODO DE ATENTIMENTO E MUITO RUIM, MUITO DEMORADO PARA VC SE COMUNICAR, E NAO AJUDOU EM NADA, SAO DESPREPARADOS, PARA ATENTIMENTO</t>
+  </si>
+  <si>
+    <t>Demora pea manutenção,  e eu solicitei a troca do equipamento,  nao fui atendida</t>
+  </si>
+  <si>
+    <t>Porque eu fiquei desde de 01/04/2026 solicitando a troca do aparelho.
+Tive que comprar galão de água porque o meu aparelho não funcionava, tive que desligar várias vezes porque ele armava e desarmava várias vezes, água não gelava e as vezes o botão não funcionava aí a água ficava direto.
+Nunca tive esse péssimo atendimento de vocês, mas sempre tem a primeira vez e espero que seja a última.
+Mesmo assim muito obrigado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demorou mais de 45 dias para trocar o aparelho que não gelava , trocaram todas as peças 2 vezes , 5 visitas e mais 4 que marquei e não vieram , ou seja marcadas 9 visitas , todos os técnicos diziam que tinha que trocar o aparelho , tive muita paciência , ufa …. Trocaram na 10 visita … o cliente não interessa , fizeram tudo para eu desistir , venci .. </t>
+  </si>
+  <si>
+    <t>O técnico marcou e nao foi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estou a duas semanas sem o purificador estar funcionando </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pela segunda vez e agendado um horário e o mesmo não é cumprido.
+Foi marcado para o período </t>
+  </si>
+  <si>
+    <t>Problema não foi resolvido. Filtro continua vazando...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O problema nos botões não foi resolvido. O técnico trocou e ficou ainda pior...desisto. Irei solicitar o cancelamento do serviço. </t>
+  </si>
+  <si>
+    <t>Não trocou a vela sob a alegação de que a vela está boa apartir do teste da água. Então, vamos ter que consumir uma água ruim pra vela ser trocada?</t>
+  </si>
+  <si>
+    <t>Eu expliquei na abertura do chamado que precisamos trocar a conexão do filtro com a água. Depois de 4 agendamentos sem sucesso, o técnico apareceu hoje e disse que só troca vela. Foi embora sem resolver nada. É um absurdo o descaso dos prestadores no Rio de Janeiro. Se acontecer um vazamento por causa disso, a Brastemp vai arcar com os custos de manutenção no imóvel?? Decepcionada. Vou abrir uma reclamação na ouvidoria agora.</t>
+  </si>
+  <si>
+    <t>Colocaram um purificador ruim com a câmara  estragada há muito usada , bebi água suja esse tempo q foi instalado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Técnico não compareceu, ninguém me procurou para remarcar a manutenção. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não voltaram para resolver o problema </t>
+  </si>
+  <si>
+    <t>Nunca vem no horário combinado!!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não resolve nenhum problema </t>
+  </si>
+  <si>
+    <t>Recebi a lavadoura amassada e foi um parto tentando realizar a troca tanta burocracia e tb o pedido de recuperação judicial que desisti de fazer a troca</t>
+  </si>
+  <si>
+    <t>Inúmeros problemas com essa empresa, já estive para cancelar 2x e fui convencida a manter. Depois de 3 semanas,  falta de técnico, técnico com OS errada, solicitei reinstalação e manutenção, e hoje, o técnico, que sabe o que faz, estava preparado apenas para reinstalar. Terei que esperar mais tempo para usar o filtro.
+Faz 3 meses que o filtro ficou parado por uma reforma na cozinha. As pesquisas e as opções de menu no WhatsApp,  por ex, são péssimas, não há a opção reinstalar, o equipamento ficou sem uso muito tempo,  etc. Estou nando essa nota porque a empresa não tem boa comunicação com os funcionários. No geral, eles são bons, mas o atendimento é segmentado e só no meu caso, erraram muito duas vezes e a terceira foi por falta, sem comunicar o cliente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Satisfação </t>
+  </si>
+  <si>
+    <t>O tecnico reparou apenas uma parte do solicitado, o fluxo de agua, porem o vazamento ele falou que o tecnico anterior tinha deixado sujeira e por isso estava congelando, mas nao limpou nem resolveu o problema, o filtro continua vazando</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não trocaram o filtro da máquina, mesmo informando que a água está com um gosto ruim, não entendi para que se marca uma visita de manutenção e não trocam no mínimo o filtro? </t>
+  </si>
+  <si>
+    <t>NÃO RECOMENDO A NINGUÉM , mais uma vez o agendamento não foi cumprido , VCS NÃO APARECEM , e mentiram dizendo que tinham ido e não tinha ninguém em casa quando eu estava em casa aguardando . Sem contar que o meu filtro já está há quase 8 MESES SEM MANUTENÇÃO.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Por motivo de só ter agenda para 3 dias após meu contato e ficar sem agua esse tempo todo,
+é um absurdo. </t>
+  </si>
+  <si>
+    <t>Visita marcada, porém o funcionário não apareceu.</t>
+  </si>
+  <si>
+    <t>Nao compensa manter o aluguel do aparelho, o melhor e comprar, existem varios produtos de excelente qualidade. Eu mesma ja estava p cancelar... provavelmente depois do meu acordo de desconto... cancele.</t>
+  </si>
+  <si>
+    <t>Serviço para atendimento no momento està ruim.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Técnico atrasou muito 20 minutos Não sei se fez manutenção correta porque foi embora em menos de 10 minutos Não trocou filtro! </t>
+  </si>
+  <si>
+    <t>O filtro é perfeito, mas não consigo resolver problemas. Estou sendo cobrado em duplicidade e não consigo receber o valor que já foi cobrado (reembolso) e também não consigo deixar de ser cobrado em duplicadade, todo mês sou cobrado, todo mês eu ligo e nada acontece.</t>
+  </si>
+  <si>
+    <t>Porque o atendimento NÃO FOI REALIZADO!!!!! O técnico NÃO compareceu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Porque o aparelho deu pane elétrica faz mais de 15 dias, eu liguei pedi prioridade visto que era um problema que inviabilizava o uso, não era uma simples troca de filtro, e não levaram em consideração meu pedido. Sou cliente desde 2008, ou seja há 18 anos e esperava um atendimento diferenciado para este tipo de ocorrência. Estava esperando até que não viessem hoje porque aí iria cancelar minha assinatura.
+Trabalho com prestação de serviços e quando um cliente me procura para solucionar um problema, procuro dar prioridade, ainda mais se for um cliente antigo e fiel.  </t>
+  </si>
+  <si>
+    <t>Não resolveu o problema</t>
+  </si>
+  <si>
+    <t>tecnico se recusou a trocar o filtro</t>
+  </si>
+  <si>
+    <t>Troca</t>
+  </si>
+  <si>
+    <t>SEGURANÇA DO PRODUTO</t>
+  </si>
+  <si>
+    <t>Troca de aparelho não efetivada</t>
+  </si>
+  <si>
+    <t>Caso sem resolução</t>
+  </si>
+  <si>
+    <t>veio e não arrumou + demora/atendimento ruim</t>
+  </si>
+  <si>
+    <t>demora manutenção + troca solicitada não atendida</t>
+  </si>
+  <si>
+    <t>desde 01/04 solicitando a troca</t>
+  </si>
+  <si>
+    <t>técnicos diziam trocar + 4 visitas faltaram</t>
+  </si>
+  <si>
+    <t>técnico marcou e não foi</t>
+  </si>
+  <si>
+    <t>duas semanas sem purificador funcionando</t>
+  </si>
+  <si>
+    <t>horário agendado não é cumprido</t>
+  </si>
+  <si>
+    <t>não resolvido, filtro continua vazando</t>
+  </si>
+  <si>
+    <t>botões não resolvido, ficou pior + cancelamento</t>
+  </si>
+  <si>
+    <t>não trocou a vela após teste</t>
+  </si>
+  <si>
+    <t>pedi troca da conexão, técnico só troca vela + 4 agendamentos</t>
+  </si>
+  <si>
+    <t>purificador ruim, câmara estragada, usado</t>
+  </si>
+  <si>
+    <t>não compareceu + ninguém remarcou</t>
+  </si>
+  <si>
+    <t>não voltaram para resolver</t>
+  </si>
+  <si>
+    <t>nunca vem no horário combinado</t>
+  </si>
+  <si>
+    <t>não resolve nenhum problema</t>
+  </si>
+  <si>
+    <t>lavadora amassada + burocracia na troca</t>
+  </si>
+  <si>
+    <t>técnico com OS errada + WhatsApp ruim</t>
+  </si>
+  <si>
+    <t>satisfação</t>
+  </si>
+  <si>
+    <t>filtro continua vazando + não limpou</t>
+  </si>
+  <si>
+    <t>não trocaram o filtro, gosto ruim</t>
+  </si>
+  <si>
+    <t>não aparecem + 8 meses sem manutenção</t>
+  </si>
+  <si>
+    <t>só agenda para 3 dias depois</t>
+  </si>
+  <si>
+    <t>visita marcada, funcionário não apareceu</t>
+  </si>
+  <si>
+    <t>não compensa manter o aluguel</t>
+  </si>
+  <si>
+    <t>serviço de atendimento está ruim</t>
+  </si>
+  <si>
+    <t>menos de 10 min, não trocou filtro + atraso</t>
+  </si>
+  <si>
+    <t>cobrado em duplicidade, sem reembolso</t>
+  </si>
+  <si>
+    <t>pane há 15 dias, prioridade ignorada</t>
+  </si>
+  <si>
+    <t>não resolveu o problema</t>
+  </si>
+  <si>
+    <t>técnico se recusou a trocar o filtro</t>
   </si>
 </sst>
 </file>
@@ -10948,7 +11174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -10973,6 +11199,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -11315,7 +11547,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1681"/>
+  <dimension ref="A1:M1713"/>
   <sheetFormatPr defaultRowHeight="24" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="4" customWidth="1"/>
@@ -80255,6 +80487,1318 @@
         <v>2530</v>
       </c>
     </row>
+    <row r="1682" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1682" s="4">
+        <v>704</v>
+      </c>
+      <c r="B1682" s="9" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1682" s="4">
+        <v>166505</v>
+      </c>
+      <c r="D1682" s="2" t="s">
+        <v>3508</v>
+      </c>
+      <c r="E1682" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1682" s="9" t="s">
+        <v>3514</v>
+      </c>
+      <c r="G1682" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1682" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1682" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1682" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1682" s="4" t="s">
+        <v>3550</v>
+      </c>
+      <c r="L1682" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1682" s="9" t="s">
+        <v>2439</v>
+      </c>
+    </row>
+    <row r="1683" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1683" s="4">
+        <v>705</v>
+      </c>
+      <c r="B1683" s="9" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1683" s="4">
+        <v>168073</v>
+      </c>
+      <c r="D1683" s="2" t="s">
+        <v>3508</v>
+      </c>
+      <c r="E1683" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1683" s="9" t="s">
+        <v>3515</v>
+      </c>
+      <c r="G1683" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1683" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1683" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1683" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1683" s="4" t="s">
+        <v>3551</v>
+      </c>
+      <c r="L1683" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1683" s="9" t="s">
+        <v>2481</v>
+      </c>
+    </row>
+    <row r="1684" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1684" s="4">
+        <v>706</v>
+      </c>
+      <c r="B1684" s="9" t="s">
+        <v>3546</v>
+      </c>
+      <c r="C1684" s="4">
+        <v>153366</v>
+      </c>
+      <c r="D1684" s="2" t="s">
+        <v>3508</v>
+      </c>
+      <c r="E1684" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1684" s="10" t="s">
+        <v>3516</v>
+      </c>
+      <c r="G1684" s="4" t="s">
+        <v>3490</v>
+      </c>
+      <c r="H1684" s="4" t="s">
+        <v>3548</v>
+      </c>
+      <c r="I1684" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1684" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1684" s="4" t="s">
+        <v>3552</v>
+      </c>
+      <c r="L1684" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1684" s="9" t="s">
+        <v>2480</v>
+      </c>
+    </row>
+    <row r="1685" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1685" s="4">
+        <v>707</v>
+      </c>
+      <c r="B1685" s="9" t="s">
+        <v>3546</v>
+      </c>
+      <c r="C1685" s="4">
+        <v>163914</v>
+      </c>
+      <c r="D1685" s="2" t="s">
+        <v>3509</v>
+      </c>
+      <c r="E1685" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1685" s="9" t="s">
+        <v>3517</v>
+      </c>
+      <c r="G1685" s="4" t="s">
+        <v>3490</v>
+      </c>
+      <c r="H1685" s="4" t="s">
+        <v>3548</v>
+      </c>
+      <c r="I1685" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1685" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1685" s="4" t="s">
+        <v>3553</v>
+      </c>
+      <c r="L1685" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1685" s="9" t="s">
+        <v>2406</v>
+      </c>
+    </row>
+    <row r="1686" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1686" s="4">
+        <v>708</v>
+      </c>
+      <c r="B1686" s="9" t="s">
+        <v>1512</v>
+      </c>
+      <c r="C1686" s="4">
+        <v>156651</v>
+      </c>
+      <c r="D1686" s="2" t="s">
+        <v>3509</v>
+      </c>
+      <c r="E1686" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1686" s="9" t="s">
+        <v>3518</v>
+      </c>
+      <c r="G1686" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1686" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1686" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1686" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1686" s="4" t="s">
+        <v>3554</v>
+      </c>
+      <c r="L1686" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1686" s="9" t="s">
+        <v>2443</v>
+      </c>
+    </row>
+    <row r="1687" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1687" s="4">
+        <v>709</v>
+      </c>
+      <c r="B1687" s="9" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1687" s="4">
+        <v>168394</v>
+      </c>
+      <c r="D1687" s="2" t="s">
+        <v>3509</v>
+      </c>
+      <c r="E1687" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1687" s="9" t="s">
+        <v>3519</v>
+      </c>
+      <c r="G1687" s="4" t="s">
+        <v>3490</v>
+      </c>
+      <c r="H1687" s="4" t="s">
+        <v>3549</v>
+      </c>
+      <c r="I1687" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1687" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1687" s="4" t="s">
+        <v>3555</v>
+      </c>
+      <c r="L1687" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1687" s="9" t="s">
+        <v>2516</v>
+      </c>
+    </row>
+    <row r="1688" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1688" s="4">
+        <v>710</v>
+      </c>
+      <c r="B1688" s="9" t="s">
+        <v>1512</v>
+      </c>
+      <c r="C1688" s="4">
+        <v>155097</v>
+      </c>
+      <c r="D1688" s="2" t="s">
+        <v>3509</v>
+      </c>
+      <c r="E1688" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1688" s="9" t="s">
+        <v>3520</v>
+      </c>
+      <c r="G1688" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1688" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1688" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1688" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1688" s="4" t="s">
+        <v>3556</v>
+      </c>
+      <c r="L1688" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1688" s="9" t="s">
+        <v>2405</v>
+      </c>
+    </row>
+    <row r="1689" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1689" s="4">
+        <v>711</v>
+      </c>
+      <c r="B1689" s="9" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1689" s="4">
+        <v>163223</v>
+      </c>
+      <c r="D1689" s="2" t="s">
+        <v>3509</v>
+      </c>
+      <c r="E1689" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1689" s="9" t="s">
+        <v>3521</v>
+      </c>
+      <c r="G1689" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1689" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1689" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1689" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1689" s="4" t="s">
+        <v>3557</v>
+      </c>
+      <c r="L1689" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1689" s="9" t="s">
+        <v>2408</v>
+      </c>
+    </row>
+    <row r="1690" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1690" s="4">
+        <v>712</v>
+      </c>
+      <c r="B1690" s="9" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1690" s="4">
+        <v>170010</v>
+      </c>
+      <c r="D1690" s="2" t="s">
+        <v>3509</v>
+      </c>
+      <c r="E1690" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1690" s="9" t="s">
+        <v>3522</v>
+      </c>
+      <c r="G1690" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1690" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1690" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1690" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1690" s="4" t="s">
+        <v>3558</v>
+      </c>
+      <c r="L1690" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1690" s="9" t="s">
+        <v>2480</v>
+      </c>
+    </row>
+    <row r="1691" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1691" s="4">
+        <v>713</v>
+      </c>
+      <c r="B1691" s="9" t="s">
+        <v>1512</v>
+      </c>
+      <c r="C1691" s="4">
+        <v>153427</v>
+      </c>
+      <c r="D1691" s="2" t="s">
+        <v>3510</v>
+      </c>
+      <c r="E1691" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1691" s="9" t="s">
+        <v>3523</v>
+      </c>
+      <c r="G1691" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1691" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I1691" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1691" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1691" s="4" t="s">
+        <v>3559</v>
+      </c>
+      <c r="L1691" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1691" s="9" t="s">
+        <v>2406</v>
+      </c>
+    </row>
+    <row r="1692" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1692" s="4">
+        <v>714</v>
+      </c>
+      <c r="B1692" s="9" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1692" s="4">
+        <v>173112</v>
+      </c>
+      <c r="D1692" s="2" t="s">
+        <v>3510</v>
+      </c>
+      <c r="E1692" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1692" s="9" t="s">
+        <v>3524</v>
+      </c>
+      <c r="G1692" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1692" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="I1692" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1692" s="9" t="s">
+        <v>1338</v>
+      </c>
+      <c r="K1692" s="4" t="s">
+        <v>3560</v>
+      </c>
+      <c r="L1692" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1692" s="9" t="s">
+        <v>2406</v>
+      </c>
+    </row>
+    <row r="1693" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1693" s="4">
+        <v>715</v>
+      </c>
+      <c r="B1693" s="9" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1693" s="4">
+        <v>172045</v>
+      </c>
+      <c r="D1693" s="2" t="s">
+        <v>3510</v>
+      </c>
+      <c r="E1693" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1693" s="9" t="s">
+        <v>3525</v>
+      </c>
+      <c r="G1693" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1693" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1693" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1693" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1693" s="4" t="s">
+        <v>3561</v>
+      </c>
+      <c r="L1693" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1693" s="9" t="s">
+        <v>2484</v>
+      </c>
+    </row>
+    <row r="1694" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1694" s="4">
+        <v>716</v>
+      </c>
+      <c r="B1694" s="9" t="s">
+        <v>1512</v>
+      </c>
+      <c r="C1694" s="4">
+        <v>157679</v>
+      </c>
+      <c r="D1694" s="2" t="s">
+        <v>3510</v>
+      </c>
+      <c r="E1694" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1694" s="9" t="s">
+        <v>3526</v>
+      </c>
+      <c r="G1694" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1694" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1694" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1694" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1694" s="4" t="s">
+        <v>3562</v>
+      </c>
+      <c r="L1694" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1694" s="9" t="s">
+        <v>2443</v>
+      </c>
+    </row>
+    <row r="1695" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1695" s="4">
+        <v>717</v>
+      </c>
+      <c r="B1695" s="9" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1695" s="4">
+        <v>165293</v>
+      </c>
+      <c r="D1695" s="2" t="s">
+        <v>3510</v>
+      </c>
+      <c r="E1695" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1695" s="9" t="s">
+        <v>3527</v>
+      </c>
+      <c r="G1695" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1695" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1695" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1695" s="9" t="s">
+        <v>1338</v>
+      </c>
+      <c r="K1695" s="4" t="s">
+        <v>3563</v>
+      </c>
+      <c r="L1695" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1695" s="9" t="s">
+        <v>2530</v>
+      </c>
+    </row>
+    <row r="1696" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1696" s="4">
+        <v>718</v>
+      </c>
+      <c r="B1696" s="9" t="s">
+        <v>1512</v>
+      </c>
+      <c r="C1696" s="4">
+        <v>162009</v>
+      </c>
+      <c r="D1696" s="2" t="s">
+        <v>3510</v>
+      </c>
+      <c r="E1696" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1696" s="9" t="s">
+        <v>3528</v>
+      </c>
+      <c r="G1696" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1696" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1696" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1696" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1696" s="4" t="s">
+        <v>3564</v>
+      </c>
+      <c r="L1696" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1696" s="9" t="s">
+        <v>2443</v>
+      </c>
+    </row>
+    <row r="1697" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1697" s="4">
+        <v>719</v>
+      </c>
+      <c r="B1697" s="9" t="s">
+        <v>3547</v>
+      </c>
+      <c r="C1697" s="4">
+        <v>172154</v>
+      </c>
+      <c r="D1697" s="2" t="s">
+        <v>3510</v>
+      </c>
+      <c r="E1697" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1697" s="9" t="s">
+        <v>3529</v>
+      </c>
+      <c r="G1697" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1697" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1697" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1697" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1697" s="4" t="s">
+        <v>3565</v>
+      </c>
+      <c r="L1697" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1697" s="9" t="s">
+        <v>2439</v>
+      </c>
+    </row>
+    <row r="1698" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1698" s="4">
+        <v>720</v>
+      </c>
+      <c r="B1698" s="9" t="s">
+        <v>1512</v>
+      </c>
+      <c r="C1698" s="4">
+        <v>170452</v>
+      </c>
+      <c r="D1698" s="2" t="s">
+        <v>3510</v>
+      </c>
+      <c r="E1698" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1698" s="9" t="s">
+        <v>3530</v>
+      </c>
+      <c r="G1698" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1698" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1698" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1698" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1698" s="4" t="s">
+        <v>3566</v>
+      </c>
+      <c r="L1698" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1698" s="9" t="s">
+        <v>2439</v>
+      </c>
+    </row>
+    <row r="1699" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1699" s="4">
+        <v>721</v>
+      </c>
+      <c r="B1699" s="9" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1699" s="4">
+        <v>173339</v>
+      </c>
+      <c r="D1699" s="2" t="s">
+        <v>3511</v>
+      </c>
+      <c r="E1699" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1699" s="9" t="s">
+        <v>3531</v>
+      </c>
+      <c r="G1699" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1699" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="I1699" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1699" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1699" s="4" t="s">
+        <v>3567</v>
+      </c>
+      <c r="L1699" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1699" s="9" t="s">
+        <v>2409</v>
+      </c>
+    </row>
+    <row r="1700" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1700" s="4">
+        <v>722</v>
+      </c>
+      <c r="B1700" s="9" t="s">
+        <v>1512</v>
+      </c>
+      <c r="C1700" s="4">
+        <v>173868</v>
+      </c>
+      <c r="D1700" s="2" t="s">
+        <v>3511</v>
+      </c>
+      <c r="E1700" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1700" s="9" t="s">
+        <v>3532</v>
+      </c>
+      <c r="G1700" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1700" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1700" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1700" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1700" s="4" t="s">
+        <v>3568</v>
+      </c>
+      <c r="L1700" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1700" s="9" t="s">
+        <v>2407</v>
+      </c>
+    </row>
+    <row r="1701" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1701" s="4">
+        <v>723</v>
+      </c>
+      <c r="B1701" s="9" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1701" s="4">
+        <v>175398</v>
+      </c>
+      <c r="D1701" s="2" t="s">
+        <v>3511</v>
+      </c>
+      <c r="E1701" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1701" s="9" t="s">
+        <v>3533</v>
+      </c>
+      <c r="G1701" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1701" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1701" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1701" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1701" s="4" t="s">
+        <v>3569</v>
+      </c>
+      <c r="L1701" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1701" s="9" t="s">
+        <v>2491</v>
+      </c>
+    </row>
+    <row r="1702" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1702" s="4">
+        <v>724</v>
+      </c>
+      <c r="B1702" s="9" t="s">
+        <v>1512</v>
+      </c>
+      <c r="C1702" s="4">
+        <v>165541</v>
+      </c>
+      <c r="D1702" s="2" t="s">
+        <v>3512</v>
+      </c>
+      <c r="E1702" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1702" s="9" t="s">
+        <v>3534</v>
+      </c>
+      <c r="G1702" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1702" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I1702" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1702" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1702" s="4" t="s">
+        <v>3570</v>
+      </c>
+      <c r="L1702" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1702" s="9" t="s">
+        <v>2483</v>
+      </c>
+    </row>
+    <row r="1703" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1703" s="4">
+        <v>725</v>
+      </c>
+      <c r="B1703" s="9" t="s">
+        <v>1512</v>
+      </c>
+      <c r="C1703" s="4">
+        <v>175852</v>
+      </c>
+      <c r="D1703" s="2" t="s">
+        <v>3512</v>
+      </c>
+      <c r="E1703" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1703" s="9" t="s">
+        <v>3535</v>
+      </c>
+      <c r="G1703" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1703" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1703" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1703" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1703" s="4" t="s">
+        <v>3571</v>
+      </c>
+      <c r="L1703" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1703" s="9" t="s">
+        <v>2490</v>
+      </c>
+    </row>
+    <row r="1704" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1704" s="4">
+        <v>726</v>
+      </c>
+      <c r="B1704" s="9" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1704" s="4">
+        <v>175672</v>
+      </c>
+      <c r="D1704" s="2" t="s">
+        <v>3512</v>
+      </c>
+      <c r="E1704" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1704" s="9" t="s">
+        <v>3536</v>
+      </c>
+      <c r="G1704" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1704" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1704" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1704" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1704" s="4" t="s">
+        <v>3572</v>
+      </c>
+      <c r="L1704" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1704" s="9" t="s">
+        <v>2409</v>
+      </c>
+    </row>
+    <row r="1705" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1705" s="4">
+        <v>727</v>
+      </c>
+      <c r="B1705" s="9" t="s">
+        <v>1512</v>
+      </c>
+      <c r="C1705" s="4">
+        <v>154868</v>
+      </c>
+      <c r="D1705" s="2" t="s">
+        <v>3512</v>
+      </c>
+      <c r="E1705" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1705" s="9" t="s">
+        <v>3537</v>
+      </c>
+      <c r="G1705" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1705" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1705" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1705" s="9" t="s">
+        <v>1338</v>
+      </c>
+      <c r="K1705" s="4" t="s">
+        <v>3573</v>
+      </c>
+      <c r="L1705" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1705" s="9" t="s">
+        <v>2484</v>
+      </c>
+    </row>
+    <row r="1706" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1706" s="4">
+        <v>728</v>
+      </c>
+      <c r="B1706" s="9" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1706" s="4">
+        <v>175611</v>
+      </c>
+      <c r="D1706" s="2" t="s">
+        <v>3512</v>
+      </c>
+      <c r="E1706" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1706" s="9" t="s">
+        <v>3538</v>
+      </c>
+      <c r="G1706" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1706" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="I1706" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1706" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1706" s="4" t="s">
+        <v>3574</v>
+      </c>
+      <c r="L1706" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1706" s="9" t="s">
+        <v>2438</v>
+      </c>
+    </row>
+    <row r="1707" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1707" s="4">
+        <v>729</v>
+      </c>
+      <c r="B1707" s="9" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1707" s="4">
+        <v>167224</v>
+      </c>
+      <c r="D1707" s="2" t="s">
+        <v>3512</v>
+      </c>
+      <c r="E1707" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1707" s="9" t="s">
+        <v>3539</v>
+      </c>
+      <c r="G1707" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1707" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1707" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1707" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1707" s="4" t="s">
+        <v>3575</v>
+      </c>
+      <c r="L1707" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1707" s="9" t="s">
+        <v>2439</v>
+      </c>
+    </row>
+    <row r="1708" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1708" s="4">
+        <v>730</v>
+      </c>
+      <c r="B1708" s="9" t="s">
+        <v>1512</v>
+      </c>
+      <c r="C1708" s="4">
+        <v>156628</v>
+      </c>
+      <c r="D1708" s="2" t="s">
+        <v>3512</v>
+      </c>
+      <c r="E1708" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1708" s="9" t="s">
+        <v>3540</v>
+      </c>
+      <c r="G1708" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1708" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I1708" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1708" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1708" s="4" t="s">
+        <v>3576</v>
+      </c>
+      <c r="L1708" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1708" s="9" t="s">
+        <v>2524</v>
+      </c>
+    </row>
+    <row r="1709" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1709" s="4">
+        <v>731</v>
+      </c>
+      <c r="B1709" s="9" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1709" s="4">
+        <v>175419</v>
+      </c>
+      <c r="D1709" s="2" t="s">
+        <v>3512</v>
+      </c>
+      <c r="E1709" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1709" s="9" t="s">
+        <v>3541</v>
+      </c>
+      <c r="G1709" s="4" t="s">
+        <v>3386</v>
+      </c>
+      <c r="H1709" s="4" t="s">
+        <v>3387</v>
+      </c>
+      <c r="I1709" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1709" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1709" s="4" t="s">
+        <v>3577</v>
+      </c>
+      <c r="L1709" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1709" s="9" t="s">
+        <v>2488</v>
+      </c>
+    </row>
+    <row r="1710" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1710" s="4">
+        <v>732</v>
+      </c>
+      <c r="B1710" s="9" t="s">
+        <v>1512</v>
+      </c>
+      <c r="C1710" s="4">
+        <v>157288</v>
+      </c>
+      <c r="D1710" s="2" t="s">
+        <v>3512</v>
+      </c>
+      <c r="E1710" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1710" s="9" t="s">
+        <v>3542</v>
+      </c>
+      <c r="G1710" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1710" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="I1710" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1710" s="9" t="s">
+        <v>1338</v>
+      </c>
+      <c r="K1710" s="4" t="s">
+        <v>1566</v>
+      </c>
+      <c r="L1710" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1710" s="9" t="s">
+        <v>2406</v>
+      </c>
+    </row>
+    <row r="1711" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1711" s="4">
+        <v>733</v>
+      </c>
+      <c r="B1711" s="9" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1711" s="4">
+        <v>167665</v>
+      </c>
+      <c r="D1711" s="2" t="s">
+        <v>3512</v>
+      </c>
+      <c r="E1711" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1711" s="9" t="s">
+        <v>3543</v>
+      </c>
+      <c r="G1711" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1711" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1711" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1711" s="9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="K1711" s="4" t="s">
+        <v>3578</v>
+      </c>
+      <c r="L1711" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1711" s="9" t="s">
+        <v>2492</v>
+      </c>
+    </row>
+    <row r="1712" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1712" s="4">
+        <v>734</v>
+      </c>
+      <c r="B1712" s="9" t="s">
+        <v>1227</v>
+      </c>
+      <c r="C1712" s="4">
+        <v>163769</v>
+      </c>
+      <c r="D1712" s="2" t="s">
+        <v>3512</v>
+      </c>
+      <c r="E1712" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1712" s="9" t="s">
+        <v>3544</v>
+      </c>
+      <c r="G1712" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1712" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1712" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1712" s="9" t="s">
+        <v>1338</v>
+      </c>
+      <c r="K1712" s="4" t="s">
+        <v>3579</v>
+      </c>
+      <c r="L1712" s="4" t="s">
+        <v>1547</v>
+      </c>
+      <c r="M1712" s="9" t="s">
+        <v>2408</v>
+      </c>
+    </row>
+    <row r="1713" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1713" s="4">
+        <v>735</v>
+      </c>
+      <c r="B1713" s="9" t="s">
+        <v>1512</v>
+      </c>
+      <c r="C1713" s="4">
+        <v>151528</v>
+      </c>
+      <c r="D1713" s="2" t="s">
+        <v>3513</v>
+      </c>
+      <c r="E1713" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1713" s="9" t="s">
+        <v>3545</v>
+      </c>
+      <c r="G1713" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1713" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I1713" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="J1713" s="9" t="s">
+        <v>1338</v>
+      </c>
+      <c r="K1713" s="4" t="s">
+        <v>3580</v>
+      </c>
+      <c r="L1713" s="4" t="s">
+        <v>1546</v>
+      </c>
+      <c r="M1713" s="9" t="s">
+        <v>2521</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>